<commit_message>
cap nhat san pham ngay 22102026
</commit_message>
<xml_diff>
--- a/ocop-thang-6-nam-2026.xlsx
+++ b/ocop-thang-6-nam-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quang\Desktop\OCOP-Quang-Ngai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0688DC77-9FF0-49FC-8929-436567E5A104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A2DC54-9824-4757-A76A-559CB041F705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,9 @@
     <sheet name="thống kê 535" sheetId="1" r:id="rId1"/>
     <sheet name="535" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'535'!$A$3:$H$3</definedName>
+  </definedNames>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -5326,19 +5329,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5347,7 +5344,13 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="9" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8992,26 +8995,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="56" t="s">
         <v>1482</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="51"/>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="A2" s="57"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
     </row>
     <row r="3" spans="1:8" s="12" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
@@ -9066,10 +9069,10 @@
       <c r="B5" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="D5" s="52" t="s">
+      <c r="D5" s="50" t="s">
         <v>109</v>
       </c>
       <c r="E5" s="8" t="s">
@@ -9092,8 +9095,8 @@
       <c r="B6" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="C6" s="52"/>
-      <c r="D6" s="52"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="50"/>
       <c r="E6" s="8" t="s">
         <v>7</v>
       </c>
@@ -9114,8 +9117,8 @@
       <c r="B7" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
       <c r="E7" s="10" t="s">
         <v>6</v>
       </c>
@@ -9136,8 +9139,8 @@
       <c r="B8" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
+      <c r="C8" s="50"/>
+      <c r="D8" s="50"/>
       <c r="E8" s="8" t="s">
         <v>7</v>
       </c>
@@ -9158,10 +9161,10 @@
       <c r="B9" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="C9" s="52" t="s">
+      <c r="C9" s="50" t="s">
         <v>120</v>
       </c>
-      <c r="D9" s="52" t="s">
+      <c r="D9" s="50" t="s">
         <v>121</v>
       </c>
       <c r="E9" s="14" t="s">
@@ -9184,8 +9187,8 @@
       <c r="B10" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="52"/>
-      <c r="D10" s="52"/>
+      <c r="C10" s="50"/>
+      <c r="D10" s="50"/>
       <c r="E10" s="14" t="s">
         <v>8</v>
       </c>
@@ -9206,10 +9209,10 @@
       <c r="B11" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="C11" s="52" t="s">
+      <c r="C11" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="D11" s="52" t="s">
+      <c r="D11" s="50" t="s">
         <v>127</v>
       </c>
       <c r="E11" s="14" t="s">
@@ -9232,8 +9235,8 @@
       <c r="B12" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
+      <c r="C12" s="50"/>
+      <c r="D12" s="50"/>
       <c r="E12" s="14" t="s">
         <v>8</v>
       </c>
@@ -9254,10 +9257,10 @@
       <c r="B13" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="C13" s="52" t="s">
+      <c r="C13" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="D13" s="52" t="s">
+      <c r="D13" s="50" t="s">
         <v>131</v>
       </c>
       <c r="E13" s="8" t="s">
@@ -9280,8 +9283,8 @@
       <c r="B14" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="C14" s="52"/>
-      <c r="D14" s="52"/>
+      <c r="C14" s="50"/>
+      <c r="D14" s="50"/>
       <c r="E14" s="8" t="s">
         <v>7</v>
       </c>
@@ -9302,8 +9305,8 @@
       <c r="B15" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
+      <c r="C15" s="50"/>
+      <c r="D15" s="50"/>
       <c r="E15" s="14" t="s">
         <v>8</v>
       </c>
@@ -9324,8 +9327,8 @@
       <c r="B16" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
+      <c r="C16" s="50"/>
+      <c r="D16" s="50"/>
       <c r="E16" s="14" t="s">
         <v>8</v>
       </c>
@@ -9346,8 +9349,8 @@
       <c r="B17" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
       <c r="E17" s="10" t="s">
         <v>7</v>
       </c>
@@ -9368,8 +9371,8 @@
       <c r="B18" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="C18" s="52"/>
-      <c r="D18" s="52"/>
+      <c r="C18" s="50"/>
+      <c r="D18" s="50"/>
       <c r="E18" s="14" t="s">
         <v>8</v>
       </c>
@@ -9390,8 +9393,8 @@
       <c r="B19" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="C19" s="52"/>
-      <c r="D19" s="52"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="50"/>
       <c r="E19" s="14" t="s">
         <v>8</v>
       </c>
@@ -9412,8 +9415,8 @@
       <c r="B20" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="C20" s="52"/>
-      <c r="D20" s="52"/>
+      <c r="C20" s="50"/>
+      <c r="D20" s="50"/>
       <c r="E20" s="14" t="s">
         <v>8</v>
       </c>
@@ -9434,8 +9437,8 @@
       <c r="B21" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="C21" s="52"/>
-      <c r="D21" s="52"/>
+      <c r="C21" s="50"/>
+      <c r="D21" s="50"/>
       <c r="E21" s="14" t="s">
         <v>8</v>
       </c>
@@ -9456,10 +9459,10 @@
       <c r="B22" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="C22" s="52" t="s">
+      <c r="C22" s="50" t="s">
         <v>143</v>
       </c>
-      <c r="D22" s="52" t="s">
+      <c r="D22" s="50" t="s">
         <v>144</v>
       </c>
       <c r="E22" s="14" t="s">
@@ -9482,8 +9485,8 @@
       <c r="B23" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="C23" s="52"/>
-      <c r="D23" s="52"/>
+      <c r="C23" s="50"/>
+      <c r="D23" s="50"/>
       <c r="E23" s="14" t="s">
         <v>8</v>
       </c>
@@ -9504,8 +9507,8 @@
       <c r="B24" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
+      <c r="C24" s="50"/>
+      <c r="D24" s="50"/>
       <c r="E24" s="14" t="s">
         <v>8</v>
       </c>
@@ -9526,8 +9529,8 @@
       <c r="B25" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="C25" s="52"/>
-      <c r="D25" s="52"/>
+      <c r="C25" s="50"/>
+      <c r="D25" s="50"/>
       <c r="E25" s="14" t="s">
         <v>8</v>
       </c>
@@ -9548,8 +9551,8 @@
       <c r="B26" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
+      <c r="C26" s="50"/>
+      <c r="D26" s="50"/>
       <c r="E26" s="14" t="s">
         <v>8</v>
       </c>
@@ -9570,8 +9573,8 @@
       <c r="B27" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="50"/>
       <c r="E27" s="14" t="s">
         <v>8</v>
       </c>
@@ -9592,8 +9595,8 @@
       <c r="B28" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
+      <c r="C28" s="50"/>
+      <c r="D28" s="50"/>
       <c r="E28" s="14" t="s">
         <v>8</v>
       </c>
@@ -9614,10 +9617,10 @@
       <c r="B29" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="C29" s="52" t="s">
+      <c r="C29" s="50" t="s">
         <v>152</v>
       </c>
-      <c r="D29" s="52" t="s">
+      <c r="D29" s="50" t="s">
         <v>153</v>
       </c>
       <c r="E29" s="14" t="s">
@@ -9640,8 +9643,8 @@
       <c r="B30" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="C30" s="52"/>
-      <c r="D30" s="52"/>
+      <c r="C30" s="50"/>
+      <c r="D30" s="50"/>
       <c r="E30" s="14" t="s">
         <v>8</v>
       </c>
@@ -9662,8 +9665,8 @@
       <c r="B31" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="C31" s="52"/>
-      <c r="D31" s="52"/>
+      <c r="C31" s="50"/>
+      <c r="D31" s="50"/>
       <c r="E31" s="14" t="s">
         <v>8</v>
       </c>
@@ -9684,8 +9687,8 @@
       <c r="B32" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="C32" s="52"/>
-      <c r="D32" s="52"/>
+      <c r="C32" s="50"/>
+      <c r="D32" s="50"/>
       <c r="E32" s="14" t="s">
         <v>8</v>
       </c>
@@ -9706,8 +9709,8 @@
       <c r="B33" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="C33" s="52"/>
-      <c r="D33" s="52"/>
+      <c r="C33" s="50"/>
+      <c r="D33" s="50"/>
       <c r="E33" s="14" t="s">
         <v>8</v>
       </c>
@@ -9804,10 +9807,10 @@
       <c r="B37" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="C37" s="52" t="s">
+      <c r="C37" s="50" t="s">
         <v>168</v>
       </c>
-      <c r="D37" s="52" t="s">
+      <c r="D37" s="50" t="s">
         <v>169</v>
       </c>
       <c r="E37" s="14" t="s">
@@ -9830,8 +9833,8 @@
       <c r="B38" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="C38" s="52"/>
-      <c r="D38" s="52"/>
+      <c r="C38" s="50"/>
+      <c r="D38" s="50"/>
       <c r="E38" s="14" t="s">
         <v>8</v>
       </c>
@@ -9878,10 +9881,10 @@
       <c r="B40" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="C40" s="52" t="s">
+      <c r="C40" s="50" t="s">
         <v>177</v>
       </c>
-      <c r="D40" s="52" t="s">
+      <c r="D40" s="50" t="s">
         <v>178</v>
       </c>
       <c r="E40" s="14" t="s">
@@ -9904,8 +9907,8 @@
       <c r="B41" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="C41" s="52"/>
-      <c r="D41" s="52"/>
+      <c r="C41" s="50"/>
+      <c r="D41" s="50"/>
       <c r="E41" s="14" t="s">
         <v>8</v>
       </c>
@@ -9926,8 +9929,8 @@
       <c r="B42" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="C42" s="52"/>
-      <c r="D42" s="52"/>
+      <c r="C42" s="50"/>
+      <c r="D42" s="50"/>
       <c r="E42" s="14" t="s">
         <v>8</v>
       </c>
@@ -9974,10 +9977,10 @@
       <c r="B44" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="C44" s="52" t="s">
+      <c r="C44" s="50" t="s">
         <v>185</v>
       </c>
-      <c r="D44" s="52" t="s">
+      <c r="D44" s="50" t="s">
         <v>186</v>
       </c>
       <c r="E44" s="14" t="s">
@@ -10000,8 +10003,8 @@
       <c r="B45" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="C45" s="52"/>
-      <c r="D45" s="52"/>
+      <c r="C45" s="50"/>
+      <c r="D45" s="50"/>
       <c r="E45" s="14" t="s">
         <v>8</v>
       </c>
@@ -10150,10 +10153,10 @@
       <c r="B51" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="C51" s="52" t="s">
+      <c r="C51" s="50" t="s">
         <v>205</v>
       </c>
-      <c r="D51" s="52" t="s">
+      <c r="D51" s="50" t="s">
         <v>206</v>
       </c>
       <c r="E51" s="14" t="s">
@@ -10176,8 +10179,8 @@
       <c r="B52" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="C52" s="52"/>
-      <c r="D52" s="52"/>
+      <c r="C52" s="50"/>
+      <c r="D52" s="50"/>
       <c r="E52" s="14" t="s">
         <v>8</v>
       </c>
@@ -10198,10 +10201,10 @@
       <c r="B53" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="C53" s="52" t="s">
+      <c r="C53" s="50" t="s">
         <v>209</v>
       </c>
-      <c r="D53" s="52" t="s">
+      <c r="D53" s="50" t="s">
         <v>210</v>
       </c>
       <c r="E53" s="14" t="s">
@@ -10224,8 +10227,8 @@
       <c r="B54" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="C54" s="52"/>
-      <c r="D54" s="52"/>
+      <c r="C54" s="50"/>
+      <c r="D54" s="50"/>
       <c r="E54" s="14" t="s">
         <v>8</v>
       </c>
@@ -10296,10 +10299,10 @@
       <c r="B57" s="16" t="s">
         <v>217</v>
       </c>
-      <c r="C57" s="52" t="s">
+      <c r="C57" s="50" t="s">
         <v>218</v>
       </c>
-      <c r="D57" s="52" t="s">
+      <c r="D57" s="50" t="s">
         <v>219</v>
       </c>
       <c r="E57" s="14" t="s">
@@ -10322,8 +10325,8 @@
       <c r="B58" s="16" t="s">
         <v>220</v>
       </c>
-      <c r="C58" s="52"/>
-      <c r="D58" s="52"/>
+      <c r="C58" s="50"/>
+      <c r="D58" s="50"/>
       <c r="E58" s="14" t="s">
         <v>8</v>
       </c>
@@ -10344,8 +10347,8 @@
       <c r="B59" s="16" t="s">
         <v>221</v>
       </c>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
+      <c r="C59" s="50"/>
+      <c r="D59" s="50"/>
       <c r="E59" s="14" t="s">
         <v>8</v>
       </c>
@@ -10366,8 +10369,8 @@
       <c r="B60" s="16" t="s">
         <v>222</v>
       </c>
-      <c r="C60" s="52"/>
-      <c r="D60" s="52"/>
+      <c r="C60" s="50"/>
+      <c r="D60" s="50"/>
       <c r="E60" s="14" t="s">
         <v>8</v>
       </c>
@@ -10388,8 +10391,8 @@
       <c r="B61" s="16" t="s">
         <v>223</v>
       </c>
-      <c r="C61" s="52"/>
-      <c r="D61" s="52"/>
+      <c r="C61" s="50"/>
+      <c r="D61" s="50"/>
       <c r="E61" s="14" t="s">
         <v>8</v>
       </c>
@@ -10410,8 +10413,8 @@
       <c r="B62" s="16" t="s">
         <v>225</v>
       </c>
-      <c r="C62" s="52"/>
-      <c r="D62" s="52"/>
+      <c r="C62" s="50"/>
+      <c r="D62" s="50"/>
       <c r="E62" s="14" t="s">
         <v>8</v>
       </c>
@@ -10432,8 +10435,8 @@
       <c r="B63" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="C63" s="52"/>
-      <c r="D63" s="52"/>
+      <c r="C63" s="50"/>
+      <c r="D63" s="50"/>
       <c r="E63" s="14" t="s">
         <v>8</v>
       </c>
@@ -10454,10 +10457,10 @@
       <c r="B64" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="C64" s="53" t="s">
+      <c r="C64" s="52" t="s">
         <v>228</v>
       </c>
-      <c r="D64" s="52" t="s">
+      <c r="D64" s="50" t="s">
         <v>229</v>
       </c>
       <c r="E64" s="14" t="s">
@@ -10480,8 +10483,8 @@
       <c r="B65" s="16" t="s">
         <v>230</v>
       </c>
-      <c r="C65" s="52"/>
-      <c r="D65" s="52"/>
+      <c r="C65" s="50"/>
+      <c r="D65" s="50"/>
       <c r="E65" s="14" t="s">
         <v>8</v>
       </c>
@@ -10528,10 +10531,10 @@
       <c r="B67" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="C67" s="52" t="s">
+      <c r="C67" s="50" t="s">
         <v>235</v>
       </c>
-      <c r="D67" s="52" t="s">
+      <c r="D67" s="50" t="s">
         <v>236</v>
       </c>
       <c r="E67" s="14" t="s">
@@ -10554,8 +10557,8 @@
       <c r="B68" s="16" t="s">
         <v>237</v>
       </c>
-      <c r="C68" s="52"/>
-      <c r="D68" s="52"/>
+      <c r="C68" s="50"/>
+      <c r="D68" s="50"/>
       <c r="E68" s="14" t="s">
         <v>8</v>
       </c>
@@ -10576,10 +10579,10 @@
       <c r="B69" s="16" t="s">
         <v>238</v>
       </c>
-      <c r="C69" s="52" t="s">
+      <c r="C69" s="50" t="s">
         <v>239</v>
       </c>
-      <c r="D69" s="52" t="s">
+      <c r="D69" s="50" t="s">
         <v>240</v>
       </c>
       <c r="E69" s="14" t="s">
@@ -10602,8 +10605,8 @@
       <c r="B70" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="C70" s="52"/>
-      <c r="D70" s="52"/>
+      <c r="C70" s="50"/>
+      <c r="D70" s="50"/>
       <c r="E70" s="14" t="s">
         <v>8</v>
       </c>
@@ -10624,8 +10627,8 @@
       <c r="B71" s="16" t="s">
         <v>242</v>
       </c>
-      <c r="C71" s="52"/>
-      <c r="D71" s="52"/>
+      <c r="C71" s="50"/>
+      <c r="D71" s="50"/>
       <c r="E71" s="14" t="s">
         <v>8</v>
       </c>
@@ -10646,8 +10649,8 @@
       <c r="B72" s="16" t="s">
         <v>243</v>
       </c>
-      <c r="C72" s="52"/>
-      <c r="D72" s="52"/>
+      <c r="C72" s="50"/>
+      <c r="D72" s="50"/>
       <c r="E72" s="14" t="s">
         <v>8</v>
       </c>
@@ -10668,8 +10671,8 @@
       <c r="B73" s="16" t="s">
         <v>244</v>
       </c>
-      <c r="C73" s="52"/>
-      <c r="D73" s="52"/>
+      <c r="C73" s="50"/>
+      <c r="D73" s="50"/>
       <c r="E73" s="14" t="s">
         <v>8</v>
       </c>
@@ -10742,10 +10745,10 @@
       <c r="B76" s="16" t="s">
         <v>252</v>
       </c>
-      <c r="C76" s="52" t="s">
+      <c r="C76" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="D76" s="52" t="s">
+      <c r="D76" s="50" t="s">
         <v>254</v>
       </c>
       <c r="E76" s="14" t="s">
@@ -10768,8 +10771,8 @@
       <c r="B77" s="16" t="s">
         <v>255</v>
       </c>
-      <c r="C77" s="52"/>
-      <c r="D77" s="52"/>
+      <c r="C77" s="50"/>
+      <c r="D77" s="50"/>
       <c r="E77" s="14" t="s">
         <v>8</v>
       </c>
@@ -11046,10 +11049,10 @@
       <c r="B88" s="16" t="s">
         <v>286</v>
       </c>
-      <c r="C88" s="52" t="s">
+      <c r="C88" s="50" t="s">
         <v>287</v>
       </c>
-      <c r="D88" s="53" t="s">
+      <c r="D88" s="52" t="s">
         <v>288</v>
       </c>
       <c r="E88" s="14" t="s">
@@ -11072,8 +11075,8 @@
       <c r="B89" s="16" t="s">
         <v>289</v>
       </c>
-      <c r="C89" s="52"/>
-      <c r="D89" s="52"/>
+      <c r="C89" s="50"/>
+      <c r="D89" s="50"/>
       <c r="E89" s="14" t="s">
         <v>8</v>
       </c>
@@ -11094,10 +11097,10 @@
       <c r="B90" s="16" t="s">
         <v>290</v>
       </c>
-      <c r="C90" s="52" t="s">
+      <c r="C90" s="50" t="s">
         <v>291</v>
       </c>
-      <c r="D90" s="52" t="s">
+      <c r="D90" s="50" t="s">
         <v>292</v>
       </c>
       <c r="E90" s="14" t="s">
@@ -11120,8 +11123,8 @@
       <c r="B91" s="16" t="s">
         <v>293</v>
       </c>
-      <c r="C91" s="52"/>
-      <c r="D91" s="52"/>
+      <c r="C91" s="50"/>
+      <c r="D91" s="50"/>
       <c r="E91" s="14" t="s">
         <v>8</v>
       </c>
@@ -11318,10 +11321,10 @@
       <c r="B99" s="16" t="s">
         <v>315</v>
       </c>
-      <c r="C99" s="54" t="s">
+      <c r="C99" s="55" t="s">
         <v>316</v>
       </c>
-      <c r="D99" s="52" t="s">
+      <c r="D99" s="50" t="s">
         <v>317</v>
       </c>
       <c r="E99" s="27" t="s">
@@ -11344,8 +11347,8 @@
       <c r="B100" s="16" t="s">
         <v>319</v>
       </c>
-      <c r="C100" s="54"/>
-      <c r="D100" s="52"/>
+      <c r="C100" s="55"/>
+      <c r="D100" s="50"/>
       <c r="E100" s="27" t="s">
         <v>7</v>
       </c>
@@ -11366,8 +11369,8 @@
       <c r="B101" s="16" t="s">
         <v>320</v>
       </c>
-      <c r="C101" s="54"/>
-      <c r="D101" s="52"/>
+      <c r="C101" s="55"/>
+      <c r="D101" s="50"/>
       <c r="E101" s="27" t="s">
         <v>7</v>
       </c>
@@ -11388,8 +11391,8 @@
       <c r="B102" s="16" t="s">
         <v>321</v>
       </c>
-      <c r="C102" s="54"/>
-      <c r="D102" s="52"/>
+      <c r="C102" s="55"/>
+      <c r="D102" s="50"/>
       <c r="E102" s="27" t="s">
         <v>7</v>
       </c>
@@ -11410,8 +11413,8 @@
       <c r="B103" s="16" t="s">
         <v>322</v>
       </c>
-      <c r="C103" s="54"/>
-      <c r="D103" s="52"/>
+      <c r="C103" s="55"/>
+      <c r="D103" s="50"/>
       <c r="E103" s="27" t="s">
         <v>7</v>
       </c>
@@ -11432,10 +11435,10 @@
       <c r="B104" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="C104" s="54" t="s">
+      <c r="C104" s="55" t="s">
         <v>325</v>
       </c>
-      <c r="D104" s="52" t="s">
+      <c r="D104" s="50" t="s">
         <v>326</v>
       </c>
       <c r="E104" s="24" t="s">
@@ -11458,8 +11461,8 @@
       <c r="B105" s="23" t="s">
         <v>328</v>
       </c>
-      <c r="C105" s="54"/>
-      <c r="D105" s="52"/>
+      <c r="C105" s="55"/>
+      <c r="D105" s="50"/>
       <c r="E105" s="24" t="s">
         <v>8</v>
       </c>
@@ -11480,8 +11483,8 @@
       <c r="B106" s="23" t="s">
         <v>329</v>
       </c>
-      <c r="C106" s="54"/>
-      <c r="D106" s="52"/>
+      <c r="C106" s="55"/>
+      <c r="D106" s="50"/>
       <c r="E106" s="24" t="s">
         <v>8</v>
       </c>
@@ -11528,10 +11531,10 @@
       <c r="B108" s="16" t="s">
         <v>334</v>
       </c>
-      <c r="C108" s="52" t="s">
+      <c r="C108" s="50" t="s">
         <v>335</v>
       </c>
-      <c r="D108" s="52" t="s">
+      <c r="D108" s="50" t="s">
         <v>336</v>
       </c>
       <c r="E108" s="24" t="s">
@@ -11554,8 +11557,8 @@
       <c r="B109" s="16" t="s">
         <v>338</v>
       </c>
-      <c r="C109" s="52"/>
-      <c r="D109" s="55"/>
+      <c r="C109" s="50"/>
+      <c r="D109" s="53"/>
       <c r="E109" s="24" t="s">
         <v>8</v>
       </c>
@@ -11576,8 +11579,8 @@
       <c r="B110" s="16" t="s">
         <v>305</v>
       </c>
-      <c r="C110" s="52"/>
-      <c r="D110" s="55"/>
+      <c r="C110" s="50"/>
+      <c r="D110" s="53"/>
       <c r="E110" s="24" t="s">
         <v>8</v>
       </c>
@@ -11696,10 +11699,10 @@
       <c r="B115" s="16" t="s">
         <v>350</v>
       </c>
-      <c r="C115" s="52" t="s">
+      <c r="C115" s="50" t="s">
         <v>351</v>
       </c>
-      <c r="D115" s="52" t="s">
+      <c r="D115" s="50" t="s">
         <v>352</v>
       </c>
       <c r="E115" s="24" t="s">
@@ -11722,8 +11725,8 @@
       <c r="B116" s="16" t="s">
         <v>354</v>
       </c>
-      <c r="C116" s="52"/>
-      <c r="D116" s="52"/>
+      <c r="C116" s="50"/>
+      <c r="D116" s="50"/>
       <c r="E116" s="24" t="s">
         <v>8</v>
       </c>
@@ -11744,8 +11747,8 @@
       <c r="B117" s="16" t="s">
         <v>355</v>
       </c>
-      <c r="C117" s="52"/>
-      <c r="D117" s="52"/>
+      <c r="C117" s="50"/>
+      <c r="D117" s="50"/>
       <c r="E117" s="24" t="s">
         <v>8</v>
       </c>
@@ -11766,10 +11769,10 @@
       <c r="B118" s="16" t="s">
         <v>356</v>
       </c>
-      <c r="C118" s="52" t="s">
+      <c r="C118" s="50" t="s">
         <v>357</v>
       </c>
-      <c r="D118" s="52" t="s">
+      <c r="D118" s="50" t="s">
         <v>358</v>
       </c>
       <c r="E118" s="24" t="s">
@@ -11792,8 +11795,8 @@
       <c r="B119" s="16" t="s">
         <v>359</v>
       </c>
-      <c r="C119" s="52"/>
-      <c r="D119" s="52"/>
+      <c r="C119" s="50"/>
+      <c r="D119" s="50"/>
       <c r="E119" s="24" t="s">
         <v>8</v>
       </c>
@@ -11968,10 +11971,10 @@
       <c r="B126" s="16" t="s">
         <v>380</v>
       </c>
-      <c r="C126" s="52" t="s">
+      <c r="C126" s="50" t="s">
         <v>381</v>
       </c>
-      <c r="D126" s="52" t="s">
+      <c r="D126" s="50" t="s">
         <v>382</v>
       </c>
       <c r="E126" s="24" t="s">
@@ -11994,8 +11997,8 @@
       <c r="B127" s="16" t="s">
         <v>383</v>
       </c>
-      <c r="C127" s="52"/>
-      <c r="D127" s="52"/>
+      <c r="C127" s="50"/>
+      <c r="D127" s="50"/>
       <c r="E127" s="24" t="s">
         <v>8</v>
       </c>
@@ -12068,10 +12071,10 @@
       <c r="B130" s="16" t="s">
         <v>389</v>
       </c>
-      <c r="C130" s="52" t="s">
+      <c r="C130" s="50" t="s">
         <v>390</v>
       </c>
-      <c r="D130" s="52" t="s">
+      <c r="D130" s="50" t="s">
         <v>391</v>
       </c>
       <c r="E130" s="24" t="s">
@@ -12094,8 +12097,8 @@
       <c r="B131" s="16" t="s">
         <v>392</v>
       </c>
-      <c r="C131" s="52"/>
-      <c r="D131" s="52"/>
+      <c r="C131" s="50"/>
+      <c r="D131" s="50"/>
       <c r="E131" s="24" t="s">
         <v>8</v>
       </c>
@@ -12418,10 +12421,10 @@
       <c r="B144" s="16" t="s">
         <v>426</v>
       </c>
-      <c r="C144" s="52" t="s">
+      <c r="C144" s="50" t="s">
         <v>427</v>
       </c>
-      <c r="D144" s="53" t="s">
+      <c r="D144" s="52" t="s">
         <v>428</v>
       </c>
       <c r="E144" s="24" t="s">
@@ -12444,8 +12447,8 @@
       <c r="B145" s="16" t="s">
         <v>430</v>
       </c>
-      <c r="C145" s="52"/>
-      <c r="D145" s="52"/>
+      <c r="C145" s="50"/>
+      <c r="D145" s="50"/>
       <c r="E145" s="24" t="s">
         <v>8</v>
       </c>
@@ -12492,10 +12495,10 @@
       <c r="B147" s="16" t="s">
         <v>434</v>
       </c>
-      <c r="C147" s="52" t="s">
+      <c r="C147" s="50" t="s">
         <v>435</v>
       </c>
-      <c r="D147" s="53" t="s">
+      <c r="D147" s="52" t="s">
         <v>436</v>
       </c>
       <c r="E147" s="24" t="s">
@@ -12518,8 +12521,8 @@
       <c r="B148" s="16" t="s">
         <v>437</v>
       </c>
-      <c r="C148" s="52"/>
-      <c r="D148" s="52"/>
+      <c r="C148" s="50"/>
+      <c r="D148" s="50"/>
       <c r="E148" s="24" t="s">
         <v>8</v>
       </c>
@@ -12540,8 +12543,8 @@
       <c r="B149" s="16" t="s">
         <v>439</v>
       </c>
-      <c r="C149" s="52"/>
-      <c r="D149" s="52"/>
+      <c r="C149" s="50"/>
+      <c r="D149" s="50"/>
       <c r="E149" s="24" t="s">
         <v>8</v>
       </c>
@@ -12588,10 +12591,10 @@
       <c r="B151" s="16" t="s">
         <v>443</v>
       </c>
-      <c r="C151" s="52" t="s">
+      <c r="C151" s="50" t="s">
         <v>444</v>
       </c>
-      <c r="D151" s="53" t="s">
+      <c r="D151" s="52" t="s">
         <v>445</v>
       </c>
       <c r="E151" s="24" t="s">
@@ -12614,8 +12617,8 @@
       <c r="B152" s="9" t="s">
         <v>447</v>
       </c>
-      <c r="C152" s="52"/>
-      <c r="D152" s="52"/>
+      <c r="C152" s="50"/>
+      <c r="D152" s="50"/>
       <c r="E152" s="10" t="s">
         <v>7</v>
       </c>
@@ -12892,10 +12895,10 @@
       <c r="B163" s="16" t="s">
         <v>475</v>
       </c>
-      <c r="C163" s="52" t="s">
+      <c r="C163" s="50" t="s">
         <v>476</v>
       </c>
-      <c r="D163" s="52" t="s">
+      <c r="D163" s="50" t="s">
         <v>477</v>
       </c>
       <c r="E163" s="24" t="s">
@@ -12918,8 +12921,8 @@
       <c r="B164" s="16" t="s">
         <v>478</v>
       </c>
-      <c r="C164" s="52"/>
-      <c r="D164" s="52"/>
+      <c r="C164" s="50"/>
+      <c r="D164" s="50"/>
       <c r="E164" s="24" t="s">
         <v>8</v>
       </c>
@@ -13016,10 +13019,10 @@
       <c r="B168" s="16" t="s">
         <v>489</v>
       </c>
-      <c r="C168" s="52" t="s">
+      <c r="C168" s="50" t="s">
         <v>490</v>
       </c>
-      <c r="D168" s="52" t="s">
+      <c r="D168" s="50" t="s">
         <v>491</v>
       </c>
       <c r="E168" s="24" t="s">
@@ -13042,8 +13045,8 @@
       <c r="B169" s="16" t="s">
         <v>493</v>
       </c>
-      <c r="C169" s="52"/>
-      <c r="D169" s="52"/>
+      <c r="C169" s="50"/>
+      <c r="D169" s="50"/>
       <c r="E169" s="24" t="s">
         <v>8</v>
       </c>
@@ -13064,8 +13067,8 @@
       <c r="B170" s="16" t="s">
         <v>494</v>
       </c>
-      <c r="C170" s="52"/>
-      <c r="D170" s="52"/>
+      <c r="C170" s="50"/>
+      <c r="D170" s="50"/>
       <c r="E170" s="24" t="s">
         <v>8</v>
       </c>
@@ -13086,8 +13089,8 @@
       <c r="B171" s="16" t="s">
         <v>496</v>
       </c>
-      <c r="C171" s="52"/>
-      <c r="D171" s="52"/>
+      <c r="C171" s="50"/>
+      <c r="D171" s="50"/>
       <c r="E171" s="24" t="s">
         <v>8</v>
       </c>
@@ -13108,8 +13111,8 @@
       <c r="B172" s="16" t="s">
         <v>497</v>
       </c>
-      <c r="C172" s="52"/>
-      <c r="D172" s="52"/>
+      <c r="C172" s="50"/>
+      <c r="D172" s="50"/>
       <c r="E172" s="24" t="s">
         <v>8</v>
       </c>
@@ -13130,8 +13133,8 @@
       <c r="B173" s="16" t="s">
         <v>498</v>
       </c>
-      <c r="C173" s="52"/>
-      <c r="D173" s="52"/>
+      <c r="C173" s="50"/>
+      <c r="D173" s="50"/>
       <c r="E173" s="24" t="s">
         <v>8</v>
       </c>
@@ -13152,8 +13155,8 @@
       <c r="B174" s="16" t="s">
         <v>500</v>
       </c>
-      <c r="C174" s="52"/>
-      <c r="D174" s="52"/>
+      <c r="C174" s="50"/>
+      <c r="D174" s="50"/>
       <c r="E174" s="24" t="s">
         <v>8</v>
       </c>
@@ -13326,10 +13329,10 @@
       <c r="B181" s="16" t="s">
         <v>517</v>
       </c>
-      <c r="C181" s="52" t="s">
+      <c r="C181" s="50" t="s">
         <v>518</v>
       </c>
-      <c r="D181" s="52" t="s">
+      <c r="D181" s="50" t="s">
         <v>519</v>
       </c>
       <c r="E181" s="24" t="s">
@@ -13352,8 +13355,8 @@
       <c r="B182" s="16" t="s">
         <v>520</v>
       </c>
-      <c r="C182" s="52"/>
-      <c r="D182" s="52"/>
+      <c r="C182" s="50"/>
+      <c r="D182" s="50"/>
       <c r="E182" s="24" t="s">
         <v>8</v>
       </c>
@@ -13374,10 +13377,10 @@
       <c r="B183" s="16" t="s">
         <v>521</v>
       </c>
-      <c r="C183" s="52" t="s">
+      <c r="C183" s="50" t="s">
         <v>522</v>
       </c>
-      <c r="D183" s="52" t="s">
+      <c r="D183" s="50" t="s">
         <v>523</v>
       </c>
       <c r="E183" s="24" t="s">
@@ -13400,8 +13403,8 @@
       <c r="B184" s="16" t="s">
         <v>524</v>
       </c>
-      <c r="C184" s="52"/>
-      <c r="D184" s="52"/>
+      <c r="C184" s="50"/>
+      <c r="D184" s="50"/>
       <c r="E184" s="24" t="s">
         <v>8</v>
       </c>
@@ -13422,8 +13425,8 @@
       <c r="B185" s="16" t="s">
         <v>525</v>
       </c>
-      <c r="C185" s="52"/>
-      <c r="D185" s="52"/>
+      <c r="C185" s="50"/>
+      <c r="D185" s="50"/>
       <c r="E185" s="24" t="s">
         <v>8</v>
       </c>
@@ -13468,10 +13471,10 @@
       <c r="B187" s="9" t="s">
         <v>528</v>
       </c>
-      <c r="C187" s="52" t="s">
+      <c r="C187" s="50" t="s">
         <v>529</v>
       </c>
-      <c r="D187" s="52" t="s">
+      <c r="D187" s="50" t="s">
         <v>530</v>
       </c>
       <c r="E187" s="28" t="s">
@@ -13494,8 +13497,8 @@
       <c r="B188" s="16" t="s">
         <v>531</v>
       </c>
-      <c r="C188" s="52"/>
-      <c r="D188" s="52"/>
+      <c r="C188" s="50"/>
+      <c r="D188" s="50"/>
       <c r="E188" s="24" t="s">
         <v>8</v>
       </c>
@@ -13516,8 +13519,8 @@
       <c r="B189" s="16" t="s">
         <v>532</v>
       </c>
-      <c r="C189" s="52"/>
-      <c r="D189" s="52"/>
+      <c r="C189" s="50"/>
+      <c r="D189" s="50"/>
       <c r="E189" s="24" t="s">
         <v>8</v>
       </c>
@@ -13664,10 +13667,10 @@
       <c r="B195" s="16" t="s">
         <v>548</v>
       </c>
-      <c r="C195" s="56" t="s">
+      <c r="C195" s="54" t="s">
         <v>549</v>
       </c>
-      <c r="D195" s="52" t="s">
+      <c r="D195" s="50" t="s">
         <v>550</v>
       </c>
       <c r="E195" s="24" t="s">
@@ -13690,8 +13693,8 @@
       <c r="B196" s="23" t="s">
         <v>552</v>
       </c>
-      <c r="C196" s="56"/>
-      <c r="D196" s="52"/>
+      <c r="C196" s="54"/>
+      <c r="D196" s="50"/>
       <c r="E196" s="24" t="s">
         <v>8</v>
       </c>
@@ -13712,8 +13715,8 @@
       <c r="B197" s="23" t="s">
         <v>554</v>
       </c>
-      <c r="C197" s="56"/>
-      <c r="D197" s="52"/>
+      <c r="C197" s="54"/>
+      <c r="D197" s="50"/>
       <c r="E197" s="24" t="s">
         <v>8</v>
       </c>
@@ -13734,8 +13737,8 @@
       <c r="B198" s="23" t="s">
         <v>556</v>
       </c>
-      <c r="C198" s="56"/>
-      <c r="D198" s="52"/>
+      <c r="C198" s="54"/>
+      <c r="D198" s="50"/>
       <c r="E198" s="24" t="s">
         <v>8</v>
       </c>
@@ -13782,10 +13785,10 @@
       <c r="B200" s="16" t="s">
         <v>560</v>
       </c>
-      <c r="C200" s="52" t="s">
+      <c r="C200" s="50" t="s">
         <v>561</v>
       </c>
-      <c r="D200" s="52" t="s">
+      <c r="D200" s="50" t="s">
         <v>562</v>
       </c>
       <c r="E200" s="24" t="s">
@@ -13808,8 +13811,8 @@
       <c r="B201" s="16" t="s">
         <v>563</v>
       </c>
-      <c r="C201" s="52"/>
-      <c r="D201" s="52"/>
+      <c r="C201" s="50"/>
+      <c r="D201" s="50"/>
       <c r="E201" s="24" t="s">
         <v>8</v>
       </c>
@@ -13856,10 +13859,10 @@
       <c r="B203" s="16" t="s">
         <v>567</v>
       </c>
-      <c r="C203" s="52" t="s">
+      <c r="C203" s="50" t="s">
         <v>568</v>
       </c>
-      <c r="D203" s="52" t="s">
+      <c r="D203" s="50" t="s">
         <v>569</v>
       </c>
       <c r="E203" s="24" t="s">
@@ -13882,8 +13885,8 @@
       <c r="B204" s="16" t="s">
         <v>570</v>
       </c>
-      <c r="C204" s="52"/>
-      <c r="D204" s="52"/>
+      <c r="C204" s="50"/>
+      <c r="D204" s="50"/>
       <c r="E204" s="24" t="s">
         <v>8</v>
       </c>
@@ -13928,10 +13931,10 @@
       <c r="B206" s="16" t="s">
         <v>573</v>
       </c>
-      <c r="C206" s="52" t="s">
+      <c r="C206" s="50" t="s">
         <v>574</v>
       </c>
-      <c r="D206" s="52" t="s">
+      <c r="D206" s="50" t="s">
         <v>575</v>
       </c>
       <c r="E206" s="24" t="s">
@@ -13954,8 +13957,8 @@
       <c r="B207" s="16" t="s">
         <v>577</v>
       </c>
-      <c r="C207" s="52"/>
-      <c r="D207" s="52"/>
+      <c r="C207" s="50"/>
+      <c r="D207" s="50"/>
       <c r="E207" s="24" t="s">
         <v>8</v>
       </c>
@@ -14002,10 +14005,10 @@
       <c r="B209" s="16" t="s">
         <v>581</v>
       </c>
-      <c r="C209" s="52" t="s">
+      <c r="C209" s="50" t="s">
         <v>582</v>
       </c>
-      <c r="D209" s="52" t="s">
+      <c r="D209" s="50" t="s">
         <v>583</v>
       </c>
       <c r="E209" s="24" t="s">
@@ -14028,8 +14031,8 @@
       <c r="B210" s="16" t="s">
         <v>584</v>
       </c>
-      <c r="C210" s="52"/>
-      <c r="D210" s="52"/>
+      <c r="C210" s="50"/>
+      <c r="D210" s="50"/>
       <c r="E210" s="24" t="s">
         <v>8</v>
       </c>
@@ -14074,10 +14077,10 @@
       <c r="B212" s="16" t="s">
         <v>587</v>
       </c>
-      <c r="C212" s="52" t="s">
+      <c r="C212" s="50" t="s">
         <v>588</v>
       </c>
-      <c r="D212" s="52" t="s">
+      <c r="D212" s="50" t="s">
         <v>589</v>
       </c>
       <c r="E212" s="24" t="s">
@@ -14100,8 +14103,8 @@
       <c r="B213" s="16" t="s">
         <v>590</v>
       </c>
-      <c r="C213" s="52"/>
-      <c r="D213" s="52"/>
+      <c r="C213" s="50"/>
+      <c r="D213" s="50"/>
       <c r="E213" s="24" t="s">
         <v>8</v>
       </c>
@@ -14122,10 +14125,10 @@
       <c r="B214" s="16" t="s">
         <v>591</v>
       </c>
-      <c r="C214" s="52" t="s">
+      <c r="C214" s="50" t="s">
         <v>592</v>
       </c>
-      <c r="D214" s="52" t="s">
+      <c r="D214" s="50" t="s">
         <v>593</v>
       </c>
       <c r="E214" s="24" t="s">
@@ -14148,8 +14151,8 @@
       <c r="B215" s="16" t="s">
         <v>594</v>
       </c>
-      <c r="C215" s="52"/>
-      <c r="D215" s="52"/>
+      <c r="C215" s="50"/>
+      <c r="D215" s="50"/>
       <c r="E215" s="24" t="s">
         <v>8</v>
       </c>
@@ -14170,8 +14173,8 @@
       <c r="B216" s="16" t="s">
         <v>595</v>
       </c>
-      <c r="C216" s="52"/>
-      <c r="D216" s="52"/>
+      <c r="C216" s="50"/>
+      <c r="D216" s="50"/>
       <c r="E216" s="24" t="s">
         <v>8</v>
       </c>
@@ -14192,10 +14195,10 @@
       <c r="B217" s="16" t="s">
         <v>596</v>
       </c>
-      <c r="C217" s="52" t="s">
+      <c r="C217" s="50" t="s">
         <v>597</v>
       </c>
-      <c r="D217" s="52" t="s">
+      <c r="D217" s="50" t="s">
         <v>598</v>
       </c>
       <c r="E217" s="24" t="s">
@@ -14218,8 +14221,8 @@
       <c r="B218" s="16" t="s">
         <v>599</v>
       </c>
-      <c r="C218" s="52"/>
-      <c r="D218" s="52"/>
+      <c r="C218" s="50"/>
+      <c r="D218" s="50"/>
       <c r="E218" s="24" t="s">
         <v>8</v>
       </c>
@@ -14340,10 +14343,10 @@
       <c r="B223" s="16" t="s">
         <v>611</v>
       </c>
-      <c r="C223" s="52" t="s">
+      <c r="C223" s="50" t="s">
         <v>612</v>
       </c>
-      <c r="D223" s="52" t="s">
+      <c r="D223" s="50" t="s">
         <v>613</v>
       </c>
       <c r="E223" s="24" t="s">
@@ -14366,8 +14369,8 @@
       <c r="B224" s="16" t="s">
         <v>614</v>
       </c>
-      <c r="C224" s="52"/>
-      <c r="D224" s="52"/>
+      <c r="C224" s="50"/>
+      <c r="D224" s="50"/>
       <c r="E224" s="24" t="s">
         <v>8</v>
       </c>
@@ -14464,10 +14467,10 @@
       <c r="B228" s="16" t="s">
         <v>625</v>
       </c>
-      <c r="C228" s="52" t="s">
+      <c r="C228" s="50" t="s">
         <v>626</v>
       </c>
-      <c r="D228" s="52" t="s">
+      <c r="D228" s="50" t="s">
         <v>627</v>
       </c>
       <c r="E228" s="24" t="s">
@@ -14490,8 +14493,8 @@
       <c r="B229" s="16" t="s">
         <v>628</v>
       </c>
-      <c r="C229" s="52"/>
-      <c r="D229" s="52"/>
+      <c r="C229" s="50"/>
+      <c r="D229" s="50"/>
       <c r="E229" s="24" t="s">
         <v>8</v>
       </c>
@@ -14562,10 +14565,10 @@
       <c r="B232" s="16" t="s">
         <v>634</v>
       </c>
-      <c r="C232" s="52" t="s">
+      <c r="C232" s="50" t="s">
         <v>635</v>
       </c>
-      <c r="D232" s="52" t="s">
+      <c r="D232" s="50" t="s">
         <v>636</v>
       </c>
       <c r="E232" s="24" t="s">
@@ -14588,8 +14591,8 @@
       <c r="B233" s="16" t="s">
         <v>637</v>
       </c>
-      <c r="C233" s="52"/>
-      <c r="D233" s="52"/>
+      <c r="C233" s="50"/>
+      <c r="D233" s="50"/>
       <c r="E233" s="24" t="s">
         <v>8</v>
       </c>
@@ -14610,8 +14613,8 @@
       <c r="B234" s="16" t="s">
         <v>638</v>
       </c>
-      <c r="C234" s="52"/>
-      <c r="D234" s="52"/>
+      <c r="C234" s="50"/>
+      <c r="D234" s="50"/>
       <c r="E234" s="24" t="s">
         <v>8</v>
       </c>
@@ -14760,10 +14763,10 @@
       <c r="B240" s="16" t="s">
         <v>655</v>
       </c>
-      <c r="C240" s="52" t="s">
+      <c r="C240" s="50" t="s">
         <v>656</v>
       </c>
-      <c r="D240" s="52" t="s">
+      <c r="D240" s="50" t="s">
         <v>657</v>
       </c>
       <c r="E240" s="24" t="s">
@@ -14786,8 +14789,8 @@
       <c r="B241" s="9" t="s">
         <v>659</v>
       </c>
-      <c r="C241" s="52"/>
-      <c r="D241" s="52"/>
+      <c r="C241" s="50"/>
+      <c r="D241" s="50"/>
       <c r="E241" s="8" t="s">
         <v>7</v>
       </c>
@@ -14808,8 +14811,8 @@
       <c r="B242" s="16" t="s">
         <v>660</v>
       </c>
-      <c r="C242" s="52"/>
-      <c r="D242" s="52"/>
+      <c r="C242" s="50"/>
+      <c r="D242" s="50"/>
       <c r="E242" s="24" t="s">
         <v>8</v>
       </c>
@@ -14830,8 +14833,8 @@
       <c r="B243" s="16" t="s">
         <v>662</v>
       </c>
-      <c r="C243" s="52"/>
-      <c r="D243" s="52"/>
+      <c r="C243" s="50"/>
+      <c r="D243" s="50"/>
       <c r="E243" s="24" t="s">
         <v>8</v>
       </c>
@@ -14852,8 +14855,8 @@
       <c r="B244" s="16" t="s">
         <v>663</v>
       </c>
-      <c r="C244" s="52"/>
-      <c r="D244" s="52"/>
+      <c r="C244" s="50"/>
+      <c r="D244" s="50"/>
       <c r="E244" s="24" t="s">
         <v>8</v>
       </c>
@@ -14874,8 +14877,8 @@
       <c r="B245" s="16" t="s">
         <v>664</v>
       </c>
-      <c r="C245" s="52"/>
-      <c r="D245" s="52"/>
+      <c r="C245" s="50"/>
+      <c r="D245" s="50"/>
       <c r="E245" s="24" t="s">
         <v>8</v>
       </c>
@@ -14896,8 +14899,8 @@
       <c r="B246" s="16" t="s">
         <v>665</v>
       </c>
-      <c r="C246" s="52"/>
-      <c r="D246" s="52"/>
+      <c r="C246" s="50"/>
+      <c r="D246" s="50"/>
       <c r="E246" s="24" t="s">
         <v>8</v>
       </c>
@@ -14918,8 +14921,8 @@
       <c r="B247" s="16" t="s">
         <v>666</v>
       </c>
-      <c r="C247" s="52"/>
-      <c r="D247" s="52"/>
+      <c r="C247" s="50"/>
+      <c r="D247" s="50"/>
       <c r="E247" s="24" t="s">
         <v>8</v>
       </c>
@@ -14992,10 +14995,10 @@
       <c r="B250" s="16" t="s">
         <v>674</v>
       </c>
-      <c r="C250" s="52" t="s">
+      <c r="C250" s="50" t="s">
         <v>675</v>
       </c>
-      <c r="D250" s="52" t="s">
+      <c r="D250" s="50" t="s">
         <v>676</v>
       </c>
       <c r="E250" s="24" t="s">
@@ -15018,8 +15021,8 @@
       <c r="B251" s="16" t="s">
         <v>677</v>
       </c>
-      <c r="C251" s="52"/>
-      <c r="D251" s="52"/>
+      <c r="C251" s="50"/>
+      <c r="D251" s="50"/>
       <c r="E251" s="24" t="s">
         <v>8</v>
       </c>
@@ -15040,8 +15043,8 @@
       <c r="B252" s="16" t="s">
         <v>678</v>
       </c>
-      <c r="C252" s="52"/>
-      <c r="D252" s="52"/>
+      <c r="C252" s="50"/>
+      <c r="D252" s="50"/>
       <c r="E252" s="24" t="s">
         <v>8</v>
       </c>
@@ -15190,10 +15193,10 @@
       <c r="B258" s="16" t="s">
         <v>695</v>
       </c>
-      <c r="C258" s="52" t="s">
+      <c r="C258" s="50" t="s">
         <v>696</v>
       </c>
-      <c r="D258" s="52" t="s">
+      <c r="D258" s="50" t="s">
         <v>697</v>
       </c>
       <c r="E258" s="24" t="s">
@@ -15216,8 +15219,8 @@
       <c r="B259" s="16" t="s">
         <v>698</v>
       </c>
-      <c r="C259" s="52"/>
-      <c r="D259" s="52"/>
+      <c r="C259" s="50"/>
+      <c r="D259" s="50"/>
       <c r="E259" s="24" t="s">
         <v>8</v>
       </c>
@@ -15238,10 +15241,10 @@
       <c r="B260" s="16" t="s">
         <v>699</v>
       </c>
-      <c r="C260" s="52" t="s">
+      <c r="C260" s="50" t="s">
         <v>263</v>
       </c>
-      <c r="D260" s="52" t="s">
+      <c r="D260" s="50" t="s">
         <v>700</v>
       </c>
       <c r="E260" s="24" t="s">
@@ -15264,8 +15267,8 @@
       <c r="B261" s="16" t="s">
         <v>701</v>
       </c>
-      <c r="C261" s="52"/>
-      <c r="D261" s="52"/>
+      <c r="C261" s="50"/>
+      <c r="D261" s="50"/>
       <c r="E261" s="14" t="s">
         <v>8</v>
       </c>
@@ -15388,10 +15391,10 @@
       <c r="B266" s="16" t="s">
         <v>714</v>
       </c>
-      <c r="C266" s="52" t="s">
+      <c r="C266" s="50" t="s">
         <v>715</v>
       </c>
-      <c r="D266" s="52" t="s">
+      <c r="D266" s="50" t="s">
         <v>716</v>
       </c>
       <c r="E266" s="14" t="s">
@@ -15414,8 +15417,8 @@
       <c r="B267" s="16" t="s">
         <v>717</v>
       </c>
-      <c r="C267" s="52"/>
-      <c r="D267" s="52"/>
+      <c r="C267" s="50"/>
+      <c r="D267" s="50"/>
       <c r="E267" s="14" t="s">
         <v>8</v>
       </c>
@@ -15436,8 +15439,8 @@
       <c r="B268" s="16" t="s">
         <v>718</v>
       </c>
-      <c r="C268" s="52"/>
-      <c r="D268" s="52"/>
+      <c r="C268" s="50"/>
+      <c r="D268" s="50"/>
       <c r="E268" s="14" t="s">
         <v>8</v>
       </c>
@@ -15458,8 +15461,8 @@
       <c r="B269" s="16" t="s">
         <v>719</v>
       </c>
-      <c r="C269" s="52"/>
-      <c r="D269" s="52"/>
+      <c r="C269" s="50"/>
+      <c r="D269" s="50"/>
       <c r="E269" s="14" t="s">
         <v>8</v>
       </c>
@@ -15480,8 +15483,8 @@
       <c r="B270" s="16" t="s">
         <v>720</v>
       </c>
-      <c r="C270" s="52"/>
-      <c r="D270" s="52"/>
+      <c r="C270" s="50"/>
+      <c r="D270" s="50"/>
       <c r="E270" s="14" t="s">
         <v>8</v>
       </c>
@@ -15502,8 +15505,8 @@
       <c r="B271" s="16" t="s">
         <v>721</v>
       </c>
-      <c r="C271" s="52"/>
-      <c r="D271" s="52"/>
+      <c r="C271" s="50"/>
+      <c r="D271" s="50"/>
       <c r="E271" s="14" t="s">
         <v>8</v>
       </c>
@@ -15550,10 +15553,10 @@
       <c r="B273" s="16" t="s">
         <v>725</v>
       </c>
-      <c r="C273" s="52" t="s">
+      <c r="C273" s="50" t="s">
         <v>726</v>
       </c>
-      <c r="D273" s="52" t="s">
+      <c r="D273" s="50" t="s">
         <v>727</v>
       </c>
       <c r="E273" s="14" t="s">
@@ -15576,8 +15579,8 @@
       <c r="B274" s="16" t="s">
         <v>728</v>
       </c>
-      <c r="C274" s="52"/>
-      <c r="D274" s="52"/>
+      <c r="C274" s="50"/>
+      <c r="D274" s="50"/>
       <c r="E274" s="14" t="s">
         <v>8</v>
       </c>
@@ -15648,10 +15651,10 @@
       <c r="B277" s="16" t="s">
         <v>734</v>
       </c>
-      <c r="C277" s="52" t="s">
+      <c r="C277" s="50" t="s">
         <v>735</v>
       </c>
-      <c r="D277" s="52" t="s">
+      <c r="D277" s="50" t="s">
         <v>736</v>
       </c>
       <c r="E277" s="14" t="s">
@@ -15674,8 +15677,8 @@
       <c r="B278" s="16" t="s">
         <v>737</v>
       </c>
-      <c r="C278" s="52"/>
-      <c r="D278" s="55"/>
+      <c r="C278" s="50"/>
+      <c r="D278" s="53"/>
       <c r="E278" s="14" t="s">
         <v>8</v>
       </c>
@@ -15696,10 +15699,10 @@
       <c r="B279" s="16" t="s">
         <v>734</v>
       </c>
-      <c r="C279" s="52" t="s">
+      <c r="C279" s="50" t="s">
         <v>738</v>
       </c>
-      <c r="D279" s="52" t="s">
+      <c r="D279" s="50" t="s">
         <v>739</v>
       </c>
       <c r="E279" s="14" t="s">
@@ -15722,8 +15725,8 @@
       <c r="B280" s="16" t="s">
         <v>737</v>
       </c>
-      <c r="C280" s="52"/>
-      <c r="D280" s="55"/>
+      <c r="C280" s="50"/>
+      <c r="D280" s="53"/>
       <c r="E280" s="14" t="s">
         <v>8</v>
       </c>
@@ -15744,10 +15747,10 @@
       <c r="B281" s="16" t="s">
         <v>740</v>
       </c>
-      <c r="C281" s="52" t="s">
+      <c r="C281" s="50" t="s">
         <v>741</v>
       </c>
-      <c r="D281" s="52" t="s">
+      <c r="D281" s="50" t="s">
         <v>742</v>
       </c>
       <c r="E281" s="14" t="s">
@@ -15770,8 +15773,8 @@
       <c r="B282" s="16" t="s">
         <v>743</v>
       </c>
-      <c r="C282" s="52"/>
-      <c r="D282" s="52"/>
+      <c r="C282" s="50"/>
+      <c r="D282" s="50"/>
       <c r="E282" s="14" t="s">
         <v>8</v>
       </c>
@@ -15868,10 +15871,10 @@
       <c r="B286" s="16" t="s">
         <v>752</v>
       </c>
-      <c r="C286" s="52" t="s">
+      <c r="C286" s="50" t="s">
         <v>753</v>
       </c>
-      <c r="D286" s="52" t="s">
+      <c r="D286" s="50" t="s">
         <v>754</v>
       </c>
       <c r="E286" s="14" t="s">
@@ -15894,8 +15897,8 @@
       <c r="B287" s="16" t="s">
         <v>756</v>
       </c>
-      <c r="C287" s="52"/>
-      <c r="D287" s="52"/>
+      <c r="C287" s="50"/>
+      <c r="D287" s="50"/>
       <c r="E287" s="14" t="s">
         <v>8</v>
       </c>
@@ -15916,8 +15919,8 @@
       <c r="B288" s="16" t="s">
         <v>757</v>
       </c>
-      <c r="C288" s="52"/>
-      <c r="D288" s="52"/>
+      <c r="C288" s="50"/>
+      <c r="D288" s="50"/>
       <c r="E288" s="14" t="s">
         <v>8</v>
       </c>
@@ -15938,10 +15941,10 @@
       <c r="B289" s="16" t="s">
         <v>758</v>
       </c>
-      <c r="C289" s="52" t="s">
+      <c r="C289" s="50" t="s">
         <v>759</v>
       </c>
-      <c r="D289" s="52" t="s">
+      <c r="D289" s="50" t="s">
         <v>760</v>
       </c>
       <c r="E289" s="14" t="s">
@@ -15964,8 +15967,8 @@
       <c r="B290" s="16" t="s">
         <v>762</v>
       </c>
-      <c r="C290" s="52"/>
-      <c r="D290" s="52"/>
+      <c r="C290" s="50"/>
+      <c r="D290" s="50"/>
       <c r="E290" s="14" t="s">
         <v>8</v>
       </c>
@@ -15986,8 +15989,8 @@
       <c r="B291" s="16" t="s">
         <v>763</v>
       </c>
-      <c r="C291" s="52"/>
-      <c r="D291" s="52"/>
+      <c r="C291" s="50"/>
+      <c r="D291" s="50"/>
       <c r="E291" s="14" t="s">
         <v>8</v>
       </c>
@@ -16009,7 +16012,7 @@
         <v>764</v>
       </c>
       <c r="C292" s="21"/>
-      <c r="D292" s="52"/>
+      <c r="D292" s="50"/>
       <c r="E292" s="14" t="s">
         <v>8</v>
       </c>
@@ -16030,10 +16033,10 @@
       <c r="B293" s="16" t="s">
         <v>765</v>
       </c>
-      <c r="C293" s="52" t="s">
+      <c r="C293" s="50" t="s">
         <v>766</v>
       </c>
-      <c r="D293" s="52" t="s">
+      <c r="D293" s="50" t="s">
         <v>767</v>
       </c>
       <c r="E293" s="14" t="s">
@@ -16056,8 +16059,8 @@
       <c r="B294" s="16" t="s">
         <v>769</v>
       </c>
-      <c r="C294" s="52"/>
-      <c r="D294" s="52"/>
+      <c r="C294" s="50"/>
+      <c r="D294" s="50"/>
       <c r="E294" s="14" t="s">
         <v>8</v>
       </c>
@@ -16078,8 +16081,8 @@
       <c r="B295" s="16" t="s">
         <v>770</v>
       </c>
-      <c r="C295" s="52"/>
-      <c r="D295" s="52"/>
+      <c r="C295" s="50"/>
+      <c r="D295" s="50"/>
       <c r="E295" s="14" t="s">
         <v>8</v>
       </c>
@@ -16100,8 +16103,8 @@
       <c r="B296" s="16" t="s">
         <v>772</v>
       </c>
-      <c r="C296" s="52"/>
-      <c r="D296" s="52"/>
+      <c r="C296" s="50"/>
+      <c r="D296" s="50"/>
       <c r="E296" s="14" t="s">
         <v>8</v>
       </c>
@@ -16122,10 +16125,10 @@
       <c r="B297" s="9" t="s">
         <v>773</v>
       </c>
-      <c r="C297" s="52" t="s">
+      <c r="C297" s="50" t="s">
         <v>774</v>
       </c>
-      <c r="D297" s="52" t="s">
+      <c r="D297" s="50" t="s">
         <v>775</v>
       </c>
       <c r="E297" s="8" t="s">
@@ -16148,8 +16151,8 @@
       <c r="B298" s="16" t="s">
         <v>776</v>
       </c>
-      <c r="C298" s="52"/>
-      <c r="D298" s="52"/>
+      <c r="C298" s="50"/>
+      <c r="D298" s="50"/>
       <c r="E298" s="14" t="s">
         <v>8</v>
       </c>
@@ -16170,8 +16173,8 @@
       <c r="B299" s="9" t="s">
         <v>778</v>
       </c>
-      <c r="C299" s="52"/>
-      <c r="D299" s="52"/>
+      <c r="C299" s="50"/>
+      <c r="D299" s="50"/>
       <c r="E299" s="8" t="s">
         <v>7</v>
       </c>
@@ -16192,8 +16195,8 @@
       <c r="B300" s="16" t="s">
         <v>779</v>
       </c>
-      <c r="C300" s="52"/>
-      <c r="D300" s="52"/>
+      <c r="C300" s="50"/>
+      <c r="D300" s="50"/>
       <c r="E300" s="14" t="s">
         <v>8</v>
       </c>
@@ -16214,8 +16217,8 @@
       <c r="B301" s="16" t="s">
         <v>780</v>
       </c>
-      <c r="C301" s="52"/>
-      <c r="D301" s="52"/>
+      <c r="C301" s="50"/>
+      <c r="D301" s="50"/>
       <c r="E301" s="14" t="s">
         <v>8</v>
       </c>
@@ -16236,8 +16239,8 @@
       <c r="B302" s="9" t="s">
         <v>781</v>
       </c>
-      <c r="C302" s="52"/>
-      <c r="D302" s="52"/>
+      <c r="C302" s="50"/>
+      <c r="D302" s="50"/>
       <c r="E302" s="8" t="s">
         <v>7</v>
       </c>
@@ -16258,8 +16261,8 @@
       <c r="B303" s="16" t="s">
         <v>783</v>
       </c>
-      <c r="C303" s="52"/>
-      <c r="D303" s="52"/>
+      <c r="C303" s="50"/>
+      <c r="D303" s="50"/>
       <c r="E303" s="14" t="s">
         <v>8</v>
       </c>
@@ -16280,8 +16283,8 @@
       <c r="B304" s="16" t="s">
         <v>784</v>
       </c>
-      <c r="C304" s="52"/>
-      <c r="D304" s="52"/>
+      <c r="C304" s="50"/>
+      <c r="D304" s="50"/>
       <c r="E304" s="14" t="s">
         <v>8</v>
       </c>
@@ -16326,10 +16329,10 @@
       <c r="B306" s="9" t="s">
         <v>787</v>
       </c>
-      <c r="C306" s="52" t="s">
+      <c r="C306" s="50" t="s">
         <v>788</v>
       </c>
-      <c r="D306" s="52" t="s">
+      <c r="D306" s="50" t="s">
         <v>789</v>
       </c>
       <c r="E306" s="8" t="s">
@@ -16352,8 +16355,8 @@
       <c r="B307" s="16" t="s">
         <v>790</v>
       </c>
-      <c r="C307" s="52"/>
-      <c r="D307" s="52"/>
+      <c r="C307" s="50"/>
+      <c r="D307" s="50"/>
       <c r="E307" s="14" t="s">
         <v>8</v>
       </c>
@@ -16374,10 +16377,10 @@
       <c r="B308" s="16" t="s">
         <v>791</v>
       </c>
-      <c r="C308" s="52" t="s">
+      <c r="C308" s="50" t="s">
         <v>792</v>
       </c>
-      <c r="D308" s="52" t="s">
+      <c r="D308" s="50" t="s">
         <v>793</v>
       </c>
       <c r="E308" s="14" t="s">
@@ -16400,8 +16403,8 @@
       <c r="B309" s="16" t="s">
         <v>794</v>
       </c>
-      <c r="C309" s="52"/>
-      <c r="D309" s="52"/>
+      <c r="C309" s="50"/>
+      <c r="D309" s="50"/>
       <c r="E309" s="14" t="s">
         <v>8</v>
       </c>
@@ -16546,10 +16549,10 @@
       <c r="B315" s="16" t="s">
         <v>808</v>
       </c>
-      <c r="C315" s="52" t="s">
+      <c r="C315" s="50" t="s">
         <v>809</v>
       </c>
-      <c r="D315" s="52" t="s">
+      <c r="D315" s="50" t="s">
         <v>810</v>
       </c>
       <c r="E315" s="14" t="s">
@@ -16572,8 +16575,8 @@
       <c r="B316" s="16" t="s">
         <v>812</v>
       </c>
-      <c r="C316" s="52"/>
-      <c r="D316" s="52"/>
+      <c r="C316" s="50"/>
+      <c r="D316" s="50"/>
       <c r="E316" s="14" t="s">
         <v>8</v>
       </c>
@@ -16670,10 +16673,10 @@
       <c r="B320" s="16" t="s">
         <v>823</v>
       </c>
-      <c r="C320" s="52" t="s">
+      <c r="C320" s="50" t="s">
         <v>824</v>
       </c>
-      <c r="D320" s="52" t="s">
+      <c r="D320" s="50" t="s">
         <v>825</v>
       </c>
       <c r="E320" s="14" t="s">
@@ -16696,8 +16699,8 @@
       <c r="B321" s="16" t="s">
         <v>826</v>
       </c>
-      <c r="C321" s="52"/>
-      <c r="D321" s="52"/>
+      <c r="C321" s="50"/>
+      <c r="D321" s="50"/>
       <c r="E321" s="14" t="s">
         <v>8</v>
       </c>
@@ -16768,10 +16771,10 @@
       <c r="B324" s="16" t="s">
         <v>832</v>
       </c>
-      <c r="C324" s="52" t="s">
+      <c r="C324" s="50" t="s">
         <v>833</v>
       </c>
-      <c r="D324" s="52" t="s">
+      <c r="D324" s="50" t="s">
         <v>834</v>
       </c>
       <c r="E324" s="14" t="s">
@@ -16794,8 +16797,8 @@
       <c r="B325" s="16" t="s">
         <v>835</v>
       </c>
-      <c r="C325" s="52"/>
-      <c r="D325" s="52"/>
+      <c r="C325" s="50"/>
+      <c r="D325" s="50"/>
       <c r="E325" s="14" t="s">
         <v>8</v>
       </c>
@@ -16942,10 +16945,10 @@
       <c r="B331" s="16" t="s">
         <v>849</v>
       </c>
-      <c r="C331" s="52" t="s">
+      <c r="C331" s="50" t="s">
         <v>850</v>
       </c>
-      <c r="D331" s="52" t="s">
+      <c r="D331" s="50" t="s">
         <v>851</v>
       </c>
       <c r="E331" s="14" t="s">
@@ -16968,8 +16971,8 @@
       <c r="B332" s="16" t="s">
         <v>634</v>
       </c>
-      <c r="C332" s="52"/>
-      <c r="D332" s="52"/>
+      <c r="C332" s="50"/>
+      <c r="D332" s="50"/>
       <c r="E332" s="14" t="s">
         <v>8</v>
       </c>
@@ -16990,10 +16993,10 @@
       <c r="B333" s="16" t="s">
         <v>852</v>
       </c>
-      <c r="C333" s="52" t="s">
+      <c r="C333" s="50" t="s">
         <v>853</v>
       </c>
-      <c r="D333" s="52" t="s">
+      <c r="D333" s="50" t="s">
         <v>854</v>
       </c>
       <c r="E333" s="14" t="s">
@@ -17016,8 +17019,8 @@
       <c r="B334" s="16" t="s">
         <v>856</v>
       </c>
-      <c r="C334" s="52"/>
-      <c r="D334" s="52"/>
+      <c r="C334" s="50"/>
+      <c r="D334" s="50"/>
       <c r="E334" s="14" t="s">
         <v>8</v>
       </c>
@@ -17038,8 +17041,8 @@
       <c r="B335" s="16" t="s">
         <v>857</v>
       </c>
-      <c r="C335" s="52"/>
-      <c r="D335" s="52"/>
+      <c r="C335" s="50"/>
+      <c r="D335" s="50"/>
       <c r="E335" s="14" t="s">
         <v>8</v>
       </c>
@@ -17060,8 +17063,8 @@
       <c r="B336" s="16" t="s">
         <v>858</v>
       </c>
-      <c r="C336" s="52"/>
-      <c r="D336" s="52"/>
+      <c r="C336" s="50"/>
+      <c r="D336" s="50"/>
       <c r="E336" s="14" t="s">
         <v>8</v>
       </c>
@@ -17082,8 +17085,8 @@
       <c r="B337" s="16" t="s">
         <v>859</v>
       </c>
-      <c r="C337" s="52"/>
-      <c r="D337" s="52"/>
+      <c r="C337" s="50"/>
+      <c r="D337" s="50"/>
       <c r="E337" s="14" t="s">
         <v>8</v>
       </c>
@@ -17104,8 +17107,8 @@
       <c r="B338" s="16" t="s">
         <v>860</v>
       </c>
-      <c r="C338" s="52"/>
-      <c r="D338" s="52"/>
+      <c r="C338" s="50"/>
+      <c r="D338" s="50"/>
       <c r="E338" s="14" t="s">
         <v>8</v>
       </c>
@@ -17126,8 +17129,8 @@
       <c r="B339" s="16" t="s">
         <v>862</v>
       </c>
-      <c r="C339" s="52"/>
-      <c r="D339" s="52"/>
+      <c r="C339" s="50"/>
+      <c r="D339" s="50"/>
       <c r="E339" s="14" t="s">
         <v>8</v>
       </c>
@@ -17224,10 +17227,10 @@
       <c r="B343" s="16" t="s">
         <v>872</v>
       </c>
-      <c r="C343" s="52" t="s">
+      <c r="C343" s="50" t="s">
         <v>873</v>
       </c>
-      <c r="D343" s="52" t="s">
+      <c r="D343" s="50" t="s">
         <v>874</v>
       </c>
       <c r="E343" s="14" t="s">
@@ -17250,8 +17253,8 @@
       <c r="B344" s="16" t="s">
         <v>876</v>
       </c>
-      <c r="C344" s="52"/>
-      <c r="D344" s="52"/>
+      <c r="C344" s="50"/>
+      <c r="D344" s="50"/>
       <c r="E344" s="14" t="s">
         <v>8</v>
       </c>
@@ -17296,10 +17299,10 @@
       <c r="B346" s="16" t="s">
         <v>879</v>
       </c>
-      <c r="C346" s="52" t="s">
+      <c r="C346" s="50" t="s">
         <v>880</v>
       </c>
-      <c r="D346" s="52" t="s">
+      <c r="D346" s="50" t="s">
         <v>881</v>
       </c>
       <c r="E346" s="14" t="s">
@@ -17322,8 +17325,8 @@
       <c r="B347" s="16" t="s">
         <v>883</v>
       </c>
-      <c r="C347" s="52"/>
-      <c r="D347" s="52"/>
+      <c r="C347" s="50"/>
+      <c r="D347" s="50"/>
       <c r="E347" s="14" t="s">
         <v>8</v>
       </c>
@@ -17570,10 +17573,10 @@
       <c r="B357" s="16" t="s">
         <v>910</v>
       </c>
-      <c r="C357" s="52" t="s">
+      <c r="C357" s="50" t="s">
         <v>911</v>
       </c>
-      <c r="D357" s="52" t="s">
+      <c r="D357" s="50" t="s">
         <v>912</v>
       </c>
       <c r="E357" s="14" t="s">
@@ -17596,8 +17599,8 @@
       <c r="B358" s="16" t="s">
         <v>914</v>
       </c>
-      <c r="C358" s="52"/>
-      <c r="D358" s="52"/>
+      <c r="C358" s="50"/>
+      <c r="D358" s="50"/>
       <c r="E358" s="14" t="s">
         <v>8</v>
       </c>
@@ -17618,10 +17621,10 @@
       <c r="B359" s="16" t="s">
         <v>916</v>
       </c>
-      <c r="C359" s="52" t="s">
+      <c r="C359" s="50" t="s">
         <v>917</v>
       </c>
-      <c r="D359" s="52" t="s">
+      <c r="D359" s="50" t="s">
         <v>918</v>
       </c>
       <c r="E359" s="14" t="s">
@@ -17644,8 +17647,8 @@
       <c r="B360" s="16" t="s">
         <v>919</v>
       </c>
-      <c r="C360" s="52"/>
-      <c r="D360" s="52"/>
+      <c r="C360" s="50"/>
+      <c r="D360" s="50"/>
       <c r="E360" s="14" t="s">
         <v>8</v>
       </c>
@@ -17666,10 +17669,10 @@
       <c r="B361" s="16" t="s">
         <v>920</v>
       </c>
-      <c r="C361" s="52" t="s">
+      <c r="C361" s="50" t="s">
         <v>921</v>
       </c>
-      <c r="D361" s="52" t="s">
+      <c r="D361" s="50" t="s">
         <v>922</v>
       </c>
       <c r="E361" s="10" t="s">
@@ -17692,8 +17695,8 @@
       <c r="B362" s="16" t="s">
         <v>924</v>
       </c>
-      <c r="C362" s="52"/>
-      <c r="D362" s="52"/>
+      <c r="C362" s="50"/>
+      <c r="D362" s="50"/>
       <c r="E362" s="10" t="s">
         <v>7</v>
       </c>
@@ -17714,10 +17717,10 @@
       <c r="B363" s="16" t="s">
         <v>925</v>
       </c>
-      <c r="C363" s="52" t="s">
+      <c r="C363" s="50" t="s">
         <v>926</v>
       </c>
-      <c r="D363" s="52" t="s">
+      <c r="D363" s="50" t="s">
         <v>927</v>
       </c>
       <c r="E363" s="10" t="s">
@@ -17740,8 +17743,8 @@
       <c r="B364" s="16" t="s">
         <v>928</v>
       </c>
-      <c r="C364" s="52"/>
-      <c r="D364" s="52"/>
+      <c r="C364" s="50"/>
+      <c r="D364" s="50"/>
       <c r="E364" s="14" t="s">
         <v>8</v>
       </c>
@@ -17886,10 +17889,10 @@
       <c r="B370" s="16" t="s">
         <v>942</v>
       </c>
-      <c r="C370" s="52" t="s">
+      <c r="C370" s="50" t="s">
         <v>943</v>
       </c>
-      <c r="D370" s="52" t="s">
+      <c r="D370" s="50" t="s">
         <v>944</v>
       </c>
       <c r="E370" s="17" t="s">
@@ -17912,8 +17915,8 @@
       <c r="B371" s="16" t="s">
         <v>946</v>
       </c>
-      <c r="C371" s="52"/>
-      <c r="D371" s="52"/>
+      <c r="C371" s="50"/>
+      <c r="D371" s="50"/>
       <c r="E371" s="17" t="s">
         <v>8</v>
       </c>
@@ -17934,8 +17937,8 @@
       <c r="B372" s="16" t="s">
         <v>947</v>
       </c>
-      <c r="C372" s="52"/>
-      <c r="D372" s="52"/>
+      <c r="C372" s="50"/>
+      <c r="D372" s="50"/>
       <c r="E372" s="17" t="s">
         <v>8</v>
       </c>
@@ -18156,10 +18159,10 @@
       <c r="B381" s="16" t="s">
         <v>971</v>
       </c>
-      <c r="C381" s="52" t="s">
+      <c r="C381" s="50" t="s">
         <v>972</v>
       </c>
-      <c r="D381" s="52" t="s">
+      <c r="D381" s="50" t="s">
         <v>973</v>
       </c>
       <c r="E381" s="10" t="s">
@@ -18182,8 +18185,8 @@
       <c r="B382" s="16" t="s">
         <v>975</v>
       </c>
-      <c r="C382" s="52"/>
-      <c r="D382" s="55"/>
+      <c r="C382" s="50"/>
+      <c r="D382" s="53"/>
       <c r="E382" s="10" t="s">
         <v>7</v>
       </c>
@@ -18406,10 +18409,10 @@
       <c r="B391" s="16" t="s">
         <v>997</v>
       </c>
-      <c r="C391" s="52" t="s">
+      <c r="C391" s="50" t="s">
         <v>998</v>
       </c>
-      <c r="D391" s="52" t="s">
+      <c r="D391" s="50" t="s">
         <v>999</v>
       </c>
       <c r="E391" s="17" t="s">
@@ -18432,8 +18435,8 @@
       <c r="B392" s="16" t="s">
         <v>1000</v>
       </c>
-      <c r="C392" s="52"/>
-      <c r="D392" s="52"/>
+      <c r="C392" s="50"/>
+      <c r="D392" s="50"/>
       <c r="E392" s="17" t="s">
         <v>8</v>
       </c>
@@ -18454,10 +18457,10 @@
       <c r="B393" s="16" t="s">
         <v>1001</v>
       </c>
-      <c r="C393" s="52" t="s">
+      <c r="C393" s="50" t="s">
         <v>1002</v>
       </c>
-      <c r="D393" s="52" t="s">
+      <c r="D393" s="50" t="s">
         <v>1003</v>
       </c>
       <c r="E393" s="17" t="s">
@@ -18480,8 +18483,8 @@
       <c r="B394" s="16" t="s">
         <v>1004</v>
       </c>
-      <c r="C394" s="52"/>
-      <c r="D394" s="52"/>
+      <c r="C394" s="50"/>
+      <c r="D394" s="50"/>
       <c r="E394" s="17" t="s">
         <v>8</v>
       </c>
@@ -18528,10 +18531,10 @@
       <c r="B396" s="16" t="s">
         <v>1010</v>
       </c>
-      <c r="C396" s="52" t="s">
+      <c r="C396" s="50" t="s">
         <v>1011</v>
       </c>
-      <c r="D396" s="52" t="s">
+      <c r="D396" s="50" t="s">
         <v>1012</v>
       </c>
       <c r="E396" s="17" t="s">
@@ -18554,8 +18557,8 @@
       <c r="B397" s="16" t="s">
         <v>1013</v>
       </c>
-      <c r="C397" s="52"/>
-      <c r="D397" s="52"/>
+      <c r="C397" s="50"/>
+      <c r="D397" s="50"/>
       <c r="E397" s="17" t="s">
         <v>8</v>
       </c>
@@ -18576,10 +18579,10 @@
       <c r="B398" s="16" t="s">
         <v>1014</v>
       </c>
-      <c r="C398" s="52" t="s">
+      <c r="C398" s="50" t="s">
         <v>1015</v>
       </c>
-      <c r="D398" s="52" t="s">
+      <c r="D398" s="50" t="s">
         <v>1016</v>
       </c>
       <c r="E398" s="10" t="s">
@@ -18602,8 +18605,8 @@
       <c r="B399" s="16" t="s">
         <v>1018</v>
       </c>
-      <c r="C399" s="52"/>
-      <c r="D399" s="55"/>
+      <c r="C399" s="50"/>
+      <c r="D399" s="53"/>
       <c r="E399" s="10" t="s">
         <v>7</v>
       </c>
@@ -18624,8 +18627,8 @@
       <c r="B400" s="16" t="s">
         <v>1019</v>
       </c>
-      <c r="C400" s="52"/>
-      <c r="D400" s="55"/>
+      <c r="C400" s="50"/>
+      <c r="D400" s="53"/>
       <c r="E400" s="10" t="s">
         <v>7</v>
       </c>
@@ -18646,10 +18649,10 @@
       <c r="B401" s="16" t="s">
         <v>1020</v>
       </c>
-      <c r="C401" s="52" t="s">
+      <c r="C401" s="50" t="s">
         <v>1021</v>
       </c>
-      <c r="D401" s="52" t="s">
+      <c r="D401" s="50" t="s">
         <v>1022</v>
       </c>
       <c r="E401" s="10" t="s">
@@ -18672,8 +18675,8 @@
       <c r="B402" s="16" t="s">
         <v>1023</v>
       </c>
-      <c r="C402" s="52"/>
-      <c r="D402" s="52"/>
+      <c r="C402" s="50"/>
+      <c r="D402" s="50"/>
       <c r="E402" s="10" t="s">
         <v>7</v>
       </c>
@@ -18694,8 +18697,8 @@
       <c r="B403" s="16" t="s">
         <v>1024</v>
       </c>
-      <c r="C403" s="52"/>
-      <c r="D403" s="52"/>
+      <c r="C403" s="50"/>
+      <c r="D403" s="50"/>
       <c r="E403" s="10" t="s">
         <v>7</v>
       </c>
@@ -18716,8 +18719,8 @@
       <c r="B404" s="16" t="s">
         <v>1025</v>
       </c>
-      <c r="C404" s="52"/>
-      <c r="D404" s="52"/>
+      <c r="C404" s="50"/>
+      <c r="D404" s="50"/>
       <c r="E404" s="10" t="s">
         <v>7</v>
       </c>
@@ -18738,8 +18741,8 @@
       <c r="B405" s="16" t="s">
         <v>1026</v>
       </c>
-      <c r="C405" s="52"/>
-      <c r="D405" s="52"/>
+      <c r="C405" s="50"/>
+      <c r="D405" s="50"/>
       <c r="E405" s="17" t="s">
         <v>8</v>
       </c>
@@ -18886,10 +18889,10 @@
       <c r="B411" s="16" t="s">
         <v>1043</v>
       </c>
-      <c r="C411" s="52" t="s">
+      <c r="C411" s="50" t="s">
         <v>1044</v>
       </c>
-      <c r="D411" s="52" t="s">
+      <c r="D411" s="50" t="s">
         <v>1045</v>
       </c>
       <c r="E411" s="17" t="s">
@@ -18912,8 +18915,8 @@
       <c r="B412" s="16" t="s">
         <v>1047</v>
       </c>
-      <c r="C412" s="52"/>
-      <c r="D412" s="52"/>
+      <c r="C412" s="50"/>
+      <c r="D412" s="50"/>
       <c r="E412" s="17" t="s">
         <v>8</v>
       </c>
@@ -19012,10 +19015,10 @@
       <c r="B416" s="16" t="s">
         <v>1059</v>
       </c>
-      <c r="C416" s="52" t="s">
+      <c r="C416" s="50" t="s">
         <v>1060</v>
       </c>
-      <c r="D416" s="52" t="s">
+      <c r="D416" s="50" t="s">
         <v>1061</v>
       </c>
       <c r="E416" s="17" t="s">
@@ -19038,8 +19041,8 @@
       <c r="B417" s="16" t="s">
         <v>1063</v>
       </c>
-      <c r="C417" s="52"/>
-      <c r="D417" s="52"/>
+      <c r="C417" s="50"/>
+      <c r="D417" s="50"/>
       <c r="E417" s="17" t="s">
         <v>8</v>
       </c>
@@ -19060,8 +19063,8 @@
       <c r="B418" s="16" t="s">
         <v>1064</v>
       </c>
-      <c r="C418" s="52"/>
-      <c r="D418" s="52"/>
+      <c r="C418" s="50"/>
+      <c r="D418" s="50"/>
       <c r="E418" s="17" t="s">
         <v>8</v>
       </c>
@@ -19082,8 +19085,8 @@
       <c r="B419" s="16" t="s">
         <v>1065</v>
       </c>
-      <c r="C419" s="52"/>
-      <c r="D419" s="52"/>
+      <c r="C419" s="50"/>
+      <c r="D419" s="50"/>
       <c r="E419" s="17" t="s">
         <v>8</v>
       </c>
@@ -19104,8 +19107,8 @@
       <c r="B420" s="16" t="s">
         <v>1066</v>
       </c>
-      <c r="C420" s="52"/>
-      <c r="D420" s="52"/>
+      <c r="C420" s="50"/>
+      <c r="D420" s="50"/>
       <c r="E420" s="10" t="s">
         <v>7</v>
       </c>
@@ -19126,8 +19129,8 @@
       <c r="B421" s="16" t="s">
         <v>1067</v>
       </c>
-      <c r="C421" s="52"/>
-      <c r="D421" s="52"/>
+      <c r="C421" s="50"/>
+      <c r="D421" s="50"/>
       <c r="E421" s="10" t="s">
         <v>7</v>
       </c>
@@ -19148,8 +19151,8 @@
       <c r="B422" s="16" t="s">
         <v>1068</v>
       </c>
-      <c r="C422" s="52"/>
-      <c r="D422" s="52"/>
+      <c r="C422" s="50"/>
+      <c r="D422" s="50"/>
       <c r="E422" s="10" t="s">
         <v>7</v>
       </c>
@@ -19170,8 +19173,8 @@
       <c r="B423" s="16" t="s">
         <v>1069</v>
       </c>
-      <c r="C423" s="52"/>
-      <c r="D423" s="52"/>
+      <c r="C423" s="50"/>
+      <c r="D423" s="50"/>
       <c r="E423" s="10" t="s">
         <v>7</v>
       </c>
@@ -19192,8 +19195,8 @@
       <c r="B424" s="16" t="s">
         <v>1070</v>
       </c>
-      <c r="C424" s="52"/>
-      <c r="D424" s="52"/>
+      <c r="C424" s="50"/>
+      <c r="D424" s="50"/>
       <c r="E424" s="10" t="s">
         <v>7</v>
       </c>
@@ -19316,10 +19319,10 @@
       <c r="B429" s="16" t="s">
         <v>1084</v>
       </c>
-      <c r="C429" s="52" t="s">
+      <c r="C429" s="50" t="s">
         <v>1085</v>
       </c>
-      <c r="D429" s="52" t="s">
+      <c r="D429" s="50" t="s">
         <v>1086</v>
       </c>
       <c r="E429" s="17" t="s">
@@ -19342,8 +19345,8 @@
       <c r="B430" s="16" t="s">
         <v>1087</v>
       </c>
-      <c r="C430" s="52"/>
-      <c r="D430" s="55"/>
+      <c r="C430" s="50"/>
+      <c r="D430" s="53"/>
       <c r="E430" s="17" t="s">
         <v>8</v>
       </c>
@@ -19414,10 +19417,10 @@
       <c r="B433" s="16" t="s">
         <v>1094</v>
       </c>
-      <c r="C433" s="52" t="s">
+      <c r="C433" s="50" t="s">
         <v>1095</v>
       </c>
-      <c r="D433" s="52" t="s">
+      <c r="D433" s="50" t="s">
         <v>1096</v>
       </c>
       <c r="E433" s="17" t="s">
@@ -19440,8 +19443,8 @@
       <c r="B434" s="16" t="s">
         <v>1098</v>
       </c>
-      <c r="C434" s="52"/>
-      <c r="D434" s="55"/>
+      <c r="C434" s="50"/>
+      <c r="D434" s="53"/>
       <c r="E434" s="17" t="s">
         <v>8</v>
       </c>
@@ -19462,8 +19465,8 @@
       <c r="B435" s="16" t="s">
         <v>1099</v>
       </c>
-      <c r="C435" s="52"/>
-      <c r="D435" s="55"/>
+      <c r="C435" s="50"/>
+      <c r="D435" s="53"/>
       <c r="E435" s="17" t="s">
         <v>8</v>
       </c>
@@ -19484,8 +19487,8 @@
       <c r="B436" s="16" t="s">
         <v>1100</v>
       </c>
-      <c r="C436" s="52"/>
-      <c r="D436" s="55"/>
+      <c r="C436" s="50"/>
+      <c r="D436" s="53"/>
       <c r="E436" s="17" t="s">
         <v>8</v>
       </c>
@@ -19530,10 +19533,10 @@
       <c r="B438" s="16" t="s">
         <v>1103</v>
       </c>
-      <c r="C438" s="52" t="s">
+      <c r="C438" s="50" t="s">
         <v>1104</v>
       </c>
-      <c r="D438" s="52" t="s">
+      <c r="D438" s="50" t="s">
         <v>1105</v>
       </c>
       <c r="E438" s="17" t="s">
@@ -19556,8 +19559,8 @@
       <c r="B439" s="16" t="s">
         <v>1107</v>
       </c>
-      <c r="C439" s="52"/>
-      <c r="D439" s="52"/>
+      <c r="C439" s="50"/>
+      <c r="D439" s="50"/>
       <c r="E439" s="17" t="s">
         <v>8</v>
       </c>
@@ -19578,8 +19581,8 @@
       <c r="B440" s="16" t="s">
         <v>1108</v>
       </c>
-      <c r="C440" s="52"/>
-      <c r="D440" s="52"/>
+      <c r="C440" s="50"/>
+      <c r="D440" s="50"/>
       <c r="E440" s="17" t="s">
         <v>8</v>
       </c>
@@ -19600,8 +19603,8 @@
       <c r="B441" s="16" t="s">
         <v>1109</v>
       </c>
-      <c r="C441" s="52"/>
-      <c r="D441" s="52"/>
+      <c r="C441" s="50"/>
+      <c r="D441" s="50"/>
       <c r="E441" s="17" t="s">
         <v>8</v>
       </c>
@@ -19622,8 +19625,8 @@
       <c r="B442" s="16" t="s">
         <v>1110</v>
       </c>
-      <c r="C442" s="52"/>
-      <c r="D442" s="52"/>
+      <c r="C442" s="50"/>
+      <c r="D442" s="50"/>
       <c r="E442" s="17" t="s">
         <v>8</v>
       </c>
@@ -19671,10 +19674,10 @@
       <c r="B444" s="16" t="s">
         <v>1113</v>
       </c>
-      <c r="C444" s="52" t="s">
+      <c r="C444" s="50" t="s">
         <v>1114</v>
       </c>
-      <c r="D444" s="52" t="s">
+      <c r="D444" s="50" t="s">
         <v>1115</v>
       </c>
       <c r="E444" s="17" t="s">
@@ -19697,8 +19700,8 @@
       <c r="B445" s="16" t="s">
         <v>1116</v>
       </c>
-      <c r="C445" s="52"/>
-      <c r="D445" s="52"/>
+      <c r="C445" s="50"/>
+      <c r="D445" s="50"/>
       <c r="E445" s="17" t="s">
         <v>8</v>
       </c>
@@ -19769,10 +19772,10 @@
       <c r="B448" s="16" t="s">
         <v>1122</v>
       </c>
-      <c r="C448" s="52" t="s">
+      <c r="C448" s="50" t="s">
         <v>1123</v>
       </c>
-      <c r="D448" s="52" t="s">
+      <c r="D448" s="50" t="s">
         <v>1124</v>
       </c>
       <c r="E448" s="17" t="s">
@@ -19795,8 +19798,8 @@
       <c r="B449" s="16" t="s">
         <v>1126</v>
       </c>
-      <c r="C449" s="52"/>
-      <c r="D449" s="52"/>
+      <c r="C449" s="50"/>
+      <c r="D449" s="50"/>
       <c r="E449" s="17" t="s">
         <v>8</v>
       </c>
@@ -19817,8 +19820,8 @@
       <c r="B450" s="16" t="s">
         <v>1127</v>
       </c>
-      <c r="C450" s="52"/>
-      <c r="D450" s="52"/>
+      <c r="C450" s="50"/>
+      <c r="D450" s="50"/>
       <c r="E450" s="17" t="s">
         <v>8</v>
       </c>
@@ -19839,8 +19842,8 @@
       <c r="B451" s="16" t="s">
         <v>1128</v>
       </c>
-      <c r="C451" s="52"/>
-      <c r="D451" s="52"/>
+      <c r="C451" s="50"/>
+      <c r="D451" s="50"/>
       <c r="E451" s="17" t="s">
         <v>8</v>
       </c>
@@ -19861,8 +19864,8 @@
       <c r="B452" s="16" t="s">
         <v>1129</v>
       </c>
-      <c r="C452" s="52"/>
-      <c r="D452" s="52"/>
+      <c r="C452" s="50"/>
+      <c r="D452" s="50"/>
       <c r="E452" s="17" t="s">
         <v>8</v>
       </c>
@@ -19883,10 +19886,10 @@
       <c r="B453" s="9" t="s">
         <v>1130</v>
       </c>
-      <c r="C453" s="52" t="s">
+      <c r="C453" s="50" t="s">
         <v>1131</v>
       </c>
-      <c r="D453" s="52" t="s">
+      <c r="D453" s="50" t="s">
         <v>1132</v>
       </c>
       <c r="E453" s="10" t="s">
@@ -19909,8 +19912,8 @@
       <c r="B454" s="9" t="s">
         <v>1134</v>
       </c>
-      <c r="C454" s="52"/>
-      <c r="D454" s="52"/>
+      <c r="C454" s="50"/>
+      <c r="D454" s="50"/>
       <c r="E454" s="10" t="s">
         <v>7</v>
       </c>
@@ -19931,8 +19934,8 @@
       <c r="B455" s="9" t="s">
         <v>1135</v>
       </c>
-      <c r="C455" s="52"/>
-      <c r="D455" s="52"/>
+      <c r="C455" s="50"/>
+      <c r="D455" s="50"/>
       <c r="E455" s="10" t="s">
         <v>7</v>
       </c>
@@ -19953,8 +19956,8 @@
       <c r="B456" s="9" t="s">
         <v>1137</v>
       </c>
-      <c r="C456" s="52"/>
-      <c r="D456" s="52"/>
+      <c r="C456" s="50"/>
+      <c r="D456" s="50"/>
       <c r="E456" s="10" t="s">
         <v>7</v>
       </c>
@@ -19975,8 +19978,8 @@
       <c r="B457" s="9" t="s">
         <v>1138</v>
       </c>
-      <c r="C457" s="52"/>
-      <c r="D457" s="52"/>
+      <c r="C457" s="50"/>
+      <c r="D457" s="50"/>
       <c r="E457" s="10" t="s">
         <v>7</v>
       </c>
@@ -19997,8 +20000,8 @@
       <c r="B458" s="16" t="s">
         <v>1139</v>
       </c>
-      <c r="C458" s="52"/>
-      <c r="D458" s="52"/>
+      <c r="C458" s="50"/>
+      <c r="D458" s="50"/>
       <c r="E458" s="17" t="s">
         <v>8</v>
       </c>
@@ -20019,8 +20022,8 @@
       <c r="B459" s="16" t="s">
         <v>1140</v>
       </c>
-      <c r="C459" s="52"/>
-      <c r="D459" s="52"/>
+      <c r="C459" s="50"/>
+      <c r="D459" s="50"/>
       <c r="E459" s="17" t="s">
         <v>8</v>
       </c>
@@ -20041,8 +20044,8 @@
       <c r="B460" s="16" t="s">
         <v>1141</v>
       </c>
-      <c r="C460" s="52"/>
-      <c r="D460" s="52"/>
+      <c r="C460" s="50"/>
+      <c r="D460" s="50"/>
       <c r="E460" s="17" t="s">
         <v>8</v>
       </c>
@@ -20063,8 +20066,8 @@
       <c r="B461" s="16" t="s">
         <v>1142</v>
       </c>
-      <c r="C461" s="52"/>
-      <c r="D461" s="52"/>
+      <c r="C461" s="50"/>
+      <c r="D461" s="50"/>
       <c r="E461" s="17" t="s">
         <v>8</v>
       </c>
@@ -20085,8 +20088,8 @@
       <c r="B462" s="16" t="s">
         <v>1143</v>
       </c>
-      <c r="C462" s="52"/>
-      <c r="D462" s="52"/>
+      <c r="C462" s="50"/>
+      <c r="D462" s="50"/>
       <c r="E462" s="17" t="s">
         <v>8</v>
       </c>
@@ -20107,8 +20110,8 @@
       <c r="B463" s="16" t="s">
         <v>1145</v>
       </c>
-      <c r="C463" s="52"/>
-      <c r="D463" s="52"/>
+      <c r="C463" s="50"/>
+      <c r="D463" s="50"/>
       <c r="E463" s="17" t="s">
         <v>8</v>
       </c>
@@ -20255,10 +20258,10 @@
       <c r="B469" s="16" t="s">
         <v>1162</v>
       </c>
-      <c r="C469" s="52" t="s">
+      <c r="C469" s="50" t="s">
         <v>1163</v>
       </c>
-      <c r="D469" s="52" t="s">
+      <c r="D469" s="50" t="s">
         <v>1164</v>
       </c>
       <c r="E469" s="17" t="s">
@@ -20281,8 +20284,8 @@
       <c r="B470" s="16" t="s">
         <v>1166</v>
       </c>
-      <c r="C470" s="52"/>
-      <c r="D470" s="52"/>
+      <c r="C470" s="50"/>
+      <c r="D470" s="50"/>
       <c r="E470" s="17" t="s">
         <v>8</v>
       </c>
@@ -20481,10 +20484,10 @@
       <c r="B478" s="16" t="s">
         <v>1188</v>
       </c>
-      <c r="C478" s="52" t="s">
+      <c r="C478" s="50" t="s">
         <v>1189</v>
       </c>
-      <c r="D478" s="52" t="s">
+      <c r="D478" s="50" t="s">
         <v>1190</v>
       </c>
       <c r="E478" s="17" t="s">
@@ -20507,8 +20510,8 @@
       <c r="B479" s="16" t="s">
         <v>1169</v>
       </c>
-      <c r="C479" s="52"/>
-      <c r="D479" s="52"/>
+      <c r="C479" s="50"/>
+      <c r="D479" s="50"/>
       <c r="E479" s="17" t="s">
         <v>8</v>
       </c>
@@ -20529,8 +20532,8 @@
       <c r="B480" s="16" t="s">
         <v>1191</v>
       </c>
-      <c r="C480" s="52"/>
-      <c r="D480" s="52"/>
+      <c r="C480" s="50"/>
+      <c r="D480" s="50"/>
       <c r="E480" s="17" t="s">
         <v>8</v>
       </c>
@@ -20653,10 +20656,10 @@
       <c r="B485" s="16" t="s">
         <v>1204</v>
       </c>
-      <c r="C485" s="52" t="s">
+      <c r="C485" s="50" t="s">
         <v>1205</v>
       </c>
-      <c r="D485" s="52" t="s">
+      <c r="D485" s="50" t="s">
         <v>1206</v>
       </c>
       <c r="E485" s="31" t="s">
@@ -20679,8 +20682,8 @@
       <c r="B486" s="16" t="s">
         <v>1208</v>
       </c>
-      <c r="C486" s="52"/>
-      <c r="D486" s="52"/>
+      <c r="C486" s="50"/>
+      <c r="D486" s="50"/>
       <c r="E486" s="31" t="s">
         <v>8</v>
       </c>
@@ -20947,10 +20950,10 @@
       <c r="B497" s="16" t="s">
         <v>1230</v>
       </c>
-      <c r="C497" s="52" t="s">
+      <c r="C497" s="50" t="s">
         <v>1231</v>
       </c>
-      <c r="D497" s="52" t="s">
+      <c r="D497" s="50" t="s">
         <v>1232</v>
       </c>
       <c r="E497" s="31" t="s">
@@ -20973,8 +20976,8 @@
       <c r="B498" s="16" t="s">
         <v>1233</v>
       </c>
-      <c r="C498" s="52"/>
-      <c r="D498" s="52"/>
+      <c r="C498" s="50"/>
+      <c r="D498" s="50"/>
       <c r="E498" s="31" t="s">
         <v>8</v>
       </c>
@@ -21123,10 +21126,10 @@
       <c r="B504" s="16" t="s">
         <v>1249</v>
       </c>
-      <c r="C504" s="52" t="s">
+      <c r="C504" s="50" t="s">
         <v>1250</v>
       </c>
-      <c r="D504" s="52" t="s">
+      <c r="D504" s="50" t="s">
         <v>1251</v>
       </c>
       <c r="E504" s="35" t="s">
@@ -21149,8 +21152,8 @@
       <c r="B505" s="16" t="s">
         <v>1253</v>
       </c>
-      <c r="C505" s="52"/>
-      <c r="D505" s="52"/>
+      <c r="C505" s="50"/>
+      <c r="D505" s="50"/>
       <c r="E505" s="17" t="s">
         <v>8</v>
       </c>
@@ -21171,8 +21174,8 @@
       <c r="B506" s="16" t="s">
         <v>1255</v>
       </c>
-      <c r="C506" s="52"/>
-      <c r="D506" s="52"/>
+      <c r="C506" s="50"/>
+      <c r="D506" s="50"/>
       <c r="E506" s="17" t="s">
         <v>8</v>
       </c>
@@ -21193,8 +21196,8 @@
       <c r="B507" s="16" t="s">
         <v>1256</v>
       </c>
-      <c r="C507" s="52"/>
-      <c r="D507" s="52"/>
+      <c r="C507" s="50"/>
+      <c r="D507" s="50"/>
       <c r="E507" s="17" t="s">
         <v>8</v>
       </c>
@@ -21215,8 +21218,8 @@
       <c r="B508" s="16" t="s">
         <v>1257</v>
       </c>
-      <c r="C508" s="52"/>
-      <c r="D508" s="52"/>
+      <c r="C508" s="50"/>
+      <c r="D508" s="50"/>
       <c r="E508" s="17" t="s">
         <v>8</v>
       </c>
@@ -21237,8 +21240,8 @@
       <c r="B509" s="16" t="s">
         <v>1258</v>
       </c>
-      <c r="C509" s="52"/>
-      <c r="D509" s="52"/>
+      <c r="C509" s="50"/>
+      <c r="D509" s="50"/>
       <c r="E509" s="17" t="s">
         <v>8</v>
       </c>
@@ -21285,10 +21288,10 @@
       <c r="B511" s="16" t="s">
         <v>1262</v>
       </c>
-      <c r="C511" s="52" t="s">
+      <c r="C511" s="50" t="s">
         <v>1263</v>
       </c>
-      <c r="D511" s="52" t="s">
+      <c r="D511" s="50" t="s">
         <v>1261</v>
       </c>
       <c r="E511" s="17" t="s">
@@ -21311,8 +21314,8 @@
       <c r="B512" s="16" t="s">
         <v>1264</v>
       </c>
-      <c r="C512" s="52"/>
-      <c r="D512" s="52"/>
+      <c r="C512" s="50"/>
+      <c r="D512" s="50"/>
       <c r="E512" s="17" t="s">
         <v>8</v>
       </c>
@@ -21357,10 +21360,10 @@
       <c r="B514" s="16" t="s">
         <v>1267</v>
       </c>
-      <c r="C514" s="52" t="s">
+      <c r="C514" s="50" t="s">
         <v>1268</v>
       </c>
-      <c r="D514" s="52" t="s">
+      <c r="D514" s="50" t="s">
         <v>1269</v>
       </c>
       <c r="E514" s="35" t="s">
@@ -21383,8 +21386,8 @@
       <c r="B515" s="16" t="s">
         <v>1270</v>
       </c>
-      <c r="C515" s="52"/>
-      <c r="D515" s="52"/>
+      <c r="C515" s="50"/>
+      <c r="D515" s="50"/>
       <c r="E515" s="35" t="s">
         <v>8</v>
       </c>
@@ -21457,10 +21460,10 @@
       <c r="B518" s="16" t="s">
         <v>1277</v>
       </c>
-      <c r="C518" s="52" t="s">
+      <c r="C518" s="50" t="s">
         <v>1278</v>
       </c>
-      <c r="D518" s="52" t="s">
+      <c r="D518" s="50" t="s">
         <v>1279</v>
       </c>
       <c r="E518" s="17" t="s">
@@ -21483,8 +21486,8 @@
       <c r="B519" s="16" t="s">
         <v>1280</v>
       </c>
-      <c r="C519" s="52"/>
-      <c r="D519" s="52"/>
+      <c r="C519" s="50"/>
+      <c r="D519" s="50"/>
       <c r="E519" s="17" t="s">
         <v>8</v>
       </c>
@@ -21505,8 +21508,8 @@
       <c r="B520" s="16" t="s">
         <v>1281</v>
       </c>
-      <c r="C520" s="52"/>
-      <c r="D520" s="52"/>
+      <c r="C520" s="50"/>
+      <c r="D520" s="50"/>
       <c r="E520" s="17" t="s">
         <v>8</v>
       </c>
@@ -21551,10 +21554,10 @@
       <c r="B522" s="16" t="s">
         <v>1284</v>
       </c>
-      <c r="C522" s="52" t="s">
+      <c r="C522" s="50" t="s">
         <v>1285</v>
       </c>
-      <c r="D522" s="52" t="s">
+      <c r="D522" s="50" t="s">
         <v>1286</v>
       </c>
       <c r="E522" s="35" t="s">
@@ -21577,8 +21580,8 @@
       <c r="B523" s="16" t="s">
         <v>1287</v>
       </c>
-      <c r="C523" s="52"/>
-      <c r="D523" s="52"/>
+      <c r="C523" s="50"/>
+      <c r="D523" s="50"/>
       <c r="E523" s="35" t="s">
         <v>8</v>
       </c>
@@ -21649,10 +21652,10 @@
       <c r="B526" s="16" t="s">
         <v>1291</v>
       </c>
-      <c r="C526" s="52" t="s">
+      <c r="C526" s="50" t="s">
         <v>1292</v>
       </c>
-      <c r="D526" s="52" t="s">
+      <c r="D526" s="50" t="s">
         <v>1293</v>
       </c>
       <c r="E526" s="17" t="s">
@@ -21675,8 +21678,8 @@
       <c r="B527" s="16" t="s">
         <v>1295</v>
       </c>
-      <c r="C527" s="52"/>
-      <c r="D527" s="52"/>
+      <c r="C527" s="50"/>
+      <c r="D527" s="50"/>
       <c r="E527" s="17" t="s">
         <v>8</v>
       </c>
@@ -21697,8 +21700,8 @@
       <c r="B528" s="16" t="s">
         <v>1296</v>
       </c>
-      <c r="C528" s="52"/>
-      <c r="D528" s="52"/>
+      <c r="C528" s="50"/>
+      <c r="D528" s="50"/>
       <c r="E528" s="17" t="s">
         <v>8</v>
       </c>
@@ -21719,8 +21722,8 @@
       <c r="B529" s="16" t="s">
         <v>1297</v>
       </c>
-      <c r="C529" s="52"/>
-      <c r="D529" s="52"/>
+      <c r="C529" s="50"/>
+      <c r="D529" s="50"/>
       <c r="E529" s="17" t="s">
         <v>8</v>
       </c>
@@ -21741,10 +21744,10 @@
       <c r="B530" s="16" t="s">
         <v>1298</v>
       </c>
-      <c r="C530" s="52" t="s">
+      <c r="C530" s="50" t="s">
         <v>1299</v>
       </c>
-      <c r="D530" s="52" t="s">
+      <c r="D530" s="50" t="s">
         <v>1300</v>
       </c>
       <c r="E530" s="17" t="s">
@@ -21767,8 +21770,8 @@
       <c r="B531" s="16" t="s">
         <v>1302</v>
       </c>
-      <c r="C531" s="52"/>
-      <c r="D531" s="52"/>
+      <c r="C531" s="50"/>
+      <c r="D531" s="50"/>
       <c r="E531" s="17" t="s">
         <v>8</v>
       </c>
@@ -21789,8 +21792,8 @@
       <c r="B532" s="16" t="s">
         <v>1303</v>
       </c>
-      <c r="C532" s="52"/>
-      <c r="D532" s="52"/>
+      <c r="C532" s="50"/>
+      <c r="D532" s="50"/>
       <c r="E532" s="8" t="s">
         <v>7</v>
       </c>
@@ -21811,8 +21814,8 @@
       <c r="B533" s="16" t="s">
         <v>1304</v>
       </c>
-      <c r="C533" s="52"/>
-      <c r="D533" s="52"/>
+      <c r="C533" s="50"/>
+      <c r="D533" s="50"/>
       <c r="E533" s="8" t="s">
         <v>7</v>
       </c>
@@ -21833,8 +21836,8 @@
       <c r="B534" s="16" t="s">
         <v>1305</v>
       </c>
-      <c r="C534" s="52"/>
-      <c r="D534" s="52"/>
+      <c r="C534" s="50"/>
+      <c r="D534" s="50"/>
       <c r="E534" s="8" t="s">
         <v>7</v>
       </c>
@@ -21855,8 +21858,8 @@
       <c r="B535" s="16" t="s">
         <v>1306</v>
       </c>
-      <c r="C535" s="52"/>
-      <c r="D535" s="52"/>
+      <c r="C535" s="50"/>
+      <c r="D535" s="50"/>
       <c r="E535" s="8" t="s">
         <v>7</v>
       </c>
@@ -21877,10 +21880,10 @@
       <c r="B536" s="16" t="s">
         <v>1307</v>
       </c>
-      <c r="C536" s="52" t="s">
+      <c r="C536" s="50" t="s">
         <v>1308</v>
       </c>
-      <c r="D536" s="52" t="s">
+      <c r="D536" s="50" t="s">
         <v>1309</v>
       </c>
       <c r="E536" s="14" t="s">
@@ -21903,8 +21906,8 @@
       <c r="B537" s="16" t="s">
         <v>1310</v>
       </c>
-      <c r="C537" s="52"/>
-      <c r="D537" s="52"/>
+      <c r="C537" s="50"/>
+      <c r="D537" s="50"/>
       <c r="E537" s="14" t="s">
         <v>8</v>
       </c>
@@ -22001,10 +22004,10 @@
       <c r="B541" s="16" t="s">
         <v>1320</v>
       </c>
-      <c r="C541" s="52" t="s">
+      <c r="C541" s="50" t="s">
         <v>1321</v>
       </c>
-      <c r="D541" s="52" t="s">
+      <c r="D541" s="50" t="s">
         <v>1322</v>
       </c>
       <c r="E541" s="17" t="s">
@@ -22027,8 +22030,8 @@
       <c r="B542" s="16" t="s">
         <v>1325</v>
       </c>
-      <c r="C542" s="52"/>
-      <c r="D542" s="52"/>
+      <c r="C542" s="50"/>
+      <c r="D542" s="50"/>
       <c r="E542" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22177,10 +22180,10 @@
       <c r="B548" s="16" t="s">
         <v>1341</v>
       </c>
-      <c r="C548" s="52" t="s">
+      <c r="C548" s="50" t="s">
         <v>1342</v>
       </c>
-      <c r="D548" s="52" t="s">
+      <c r="D548" s="50" t="s">
         <v>1343</v>
       </c>
       <c r="E548" s="17" t="s">
@@ -22203,8 +22206,8 @@
       <c r="B549" s="16" t="s">
         <v>1344</v>
       </c>
-      <c r="C549" s="52"/>
-      <c r="D549" s="55"/>
+      <c r="C549" s="50"/>
+      <c r="D549" s="53"/>
       <c r="E549" s="17" t="s">
         <v>8</v>
       </c>
@@ -22225,8 +22228,8 @@
       <c r="B550" s="16" t="s">
         <v>1345</v>
       </c>
-      <c r="C550" s="52"/>
-      <c r="D550" s="55"/>
+      <c r="C550" s="50"/>
+      <c r="D550" s="53"/>
       <c r="E550" s="17" t="s">
         <v>8</v>
       </c>
@@ -22321,10 +22324,10 @@
       <c r="B554" s="16" t="s">
         <v>1353</v>
       </c>
-      <c r="C554" s="52" t="s">
+      <c r="C554" s="50" t="s">
         <v>1354</v>
       </c>
-      <c r="D554" s="52" t="s">
+      <c r="D554" s="50" t="s">
         <v>1355</v>
       </c>
       <c r="E554" s="17" t="s">
@@ -22347,8 +22350,8 @@
       <c r="B555" s="16" t="s">
         <v>1356</v>
       </c>
-      <c r="C555" s="52"/>
-      <c r="D555" s="52"/>
+      <c r="C555" s="50"/>
+      <c r="D555" s="50"/>
       <c r="E555" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22393,10 +22396,10 @@
       <c r="B557" s="16" t="s">
         <v>1359</v>
       </c>
-      <c r="C557" s="52" t="s">
+      <c r="C557" s="50" t="s">
         <v>1360</v>
       </c>
-      <c r="D557" s="53" t="s">
+      <c r="D557" s="52" t="s">
         <v>1361</v>
       </c>
       <c r="E557" s="17" t="s">
@@ -22419,8 +22422,8 @@
       <c r="B558" s="16" t="s">
         <v>1363</v>
       </c>
-      <c r="C558" s="52"/>
-      <c r="D558" s="53"/>
+      <c r="C558" s="50"/>
+      <c r="D558" s="52"/>
       <c r="E558" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22441,8 +22444,8 @@
       <c r="B559" s="16" t="s">
         <v>1364</v>
       </c>
-      <c r="C559" s="52"/>
-      <c r="D559" s="53"/>
+      <c r="C559" s="50"/>
+      <c r="D559" s="52"/>
       <c r="E559" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22463,8 +22466,8 @@
       <c r="B560" s="16" t="s">
         <v>1365</v>
       </c>
-      <c r="C560" s="52"/>
-      <c r="D560" s="53"/>
+      <c r="C560" s="50"/>
+      <c r="D560" s="52"/>
       <c r="E560" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22485,8 +22488,8 @@
       <c r="B561" s="16" t="s">
         <v>1366</v>
       </c>
-      <c r="C561" s="52"/>
-      <c r="D561" s="53"/>
+      <c r="C561" s="50"/>
+      <c r="D561" s="52"/>
       <c r="E561" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22507,8 +22510,8 @@
       <c r="B562" s="16" t="s">
         <v>1367</v>
       </c>
-      <c r="C562" s="52"/>
-      <c r="D562" s="53"/>
+      <c r="C562" s="50"/>
+      <c r="D562" s="52"/>
       <c r="E562" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22529,8 +22532,8 @@
       <c r="B563" s="16" t="s">
         <v>1368</v>
       </c>
-      <c r="C563" s="52"/>
-      <c r="D563" s="53"/>
+      <c r="C563" s="50"/>
+      <c r="D563" s="52"/>
       <c r="E563" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22551,8 +22554,8 @@
       <c r="B564" s="16" t="s">
         <v>1369</v>
       </c>
-      <c r="C564" s="52"/>
-      <c r="D564" s="53"/>
+      <c r="C564" s="50"/>
+      <c r="D564" s="52"/>
       <c r="E564" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22573,8 +22576,8 @@
       <c r="B565" s="16" t="s">
         <v>1370</v>
       </c>
-      <c r="C565" s="52"/>
-      <c r="D565" s="53"/>
+      <c r="C565" s="50"/>
+      <c r="D565" s="52"/>
       <c r="E565" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22595,8 +22598,8 @@
       <c r="B566" s="16" t="s">
         <v>1371</v>
       </c>
-      <c r="C566" s="52"/>
-      <c r="D566" s="53"/>
+      <c r="C566" s="50"/>
+      <c r="D566" s="52"/>
       <c r="E566" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22617,8 +22620,8 @@
       <c r="B567" s="16" t="s">
         <v>1372</v>
       </c>
-      <c r="C567" s="52"/>
-      <c r="D567" s="53"/>
+      <c r="C567" s="50"/>
+      <c r="D567" s="52"/>
       <c r="E567" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22639,8 +22642,8 @@
       <c r="B568" s="9" t="s">
         <v>1374</v>
       </c>
-      <c r="C568" s="52"/>
-      <c r="D568" s="53"/>
+      <c r="C568" s="50"/>
+      <c r="D568" s="52"/>
       <c r="E568" s="10" t="s">
         <v>7</v>
       </c>
@@ -22661,8 +22664,8 @@
       <c r="B569" s="9" t="s">
         <v>1376</v>
       </c>
-      <c r="C569" s="52"/>
-      <c r="D569" s="53"/>
+      <c r="C569" s="50"/>
+      <c r="D569" s="52"/>
       <c r="E569" s="10" t="s">
         <v>7</v>
       </c>
@@ -22683,10 +22686,10 @@
       <c r="B570" s="16" t="s">
         <v>1377</v>
       </c>
-      <c r="C570" s="52" t="s">
+      <c r="C570" s="50" t="s">
         <v>1378</v>
       </c>
-      <c r="D570" s="53" t="s">
+      <c r="D570" s="52" t="s">
         <v>1379</v>
       </c>
       <c r="E570" s="17" t="s">
@@ -22709,8 +22712,8 @@
       <c r="B571" s="16" t="s">
         <v>1380</v>
       </c>
-      <c r="C571" s="52"/>
-      <c r="D571" s="52"/>
+      <c r="C571" s="50"/>
+      <c r="D571" s="50"/>
       <c r="E571" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22731,8 +22734,8 @@
       <c r="B572" s="16" t="s">
         <v>1381</v>
       </c>
-      <c r="C572" s="52"/>
-      <c r="D572" s="52"/>
+      <c r="C572" s="50"/>
+      <c r="D572" s="50"/>
       <c r="E572" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22753,8 +22756,8 @@
       <c r="B573" s="9" t="s">
         <v>1382</v>
       </c>
-      <c r="C573" s="52"/>
-      <c r="D573" s="52"/>
+      <c r="C573" s="50"/>
+      <c r="D573" s="50"/>
       <c r="E573" s="10" t="s">
         <v>7</v>
       </c>
@@ -22775,8 +22778,8 @@
       <c r="B574" s="9" t="s">
         <v>1383</v>
       </c>
-      <c r="C574" s="52"/>
-      <c r="D574" s="52"/>
+      <c r="C574" s="50"/>
+      <c r="D574" s="50"/>
       <c r="E574" s="10" t="s">
         <v>7</v>
       </c>
@@ -22797,10 +22800,10 @@
       <c r="B575" s="16" t="s">
         <v>1384</v>
       </c>
-      <c r="C575" s="52" t="s">
+      <c r="C575" s="50" t="s">
         <v>1385</v>
       </c>
-      <c r="D575" s="52" t="s">
+      <c r="D575" s="50" t="s">
         <v>1386</v>
       </c>
       <c r="E575" s="17" t="s">
@@ -22823,8 +22826,8 @@
       <c r="B576" s="16" t="s">
         <v>1387</v>
       </c>
-      <c r="C576" s="52"/>
-      <c r="D576" s="52"/>
+      <c r="C576" s="50"/>
+      <c r="D576" s="50"/>
       <c r="E576" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22845,10 +22848,10 @@
       <c r="B577" s="16" t="s">
         <v>1388</v>
       </c>
-      <c r="C577" s="52" t="s">
+      <c r="C577" s="50" t="s">
         <v>1389</v>
       </c>
-      <c r="D577" s="57" t="s">
+      <c r="D577" s="51" t="s">
         <v>1390</v>
       </c>
       <c r="E577" s="17" t="s">
@@ -22871,8 +22874,8 @@
       <c r="B578" s="16" t="s">
         <v>1391</v>
       </c>
-      <c r="C578" s="52"/>
-      <c r="D578" s="57"/>
+      <c r="C578" s="50"/>
+      <c r="D578" s="51"/>
       <c r="E578" s="17" t="s">
         <v>1323</v>
       </c>
@@ -22971,10 +22974,10 @@
       <c r="B582" s="16" t="s">
         <v>1404</v>
       </c>
-      <c r="C582" s="52" t="s">
+      <c r="C582" s="50" t="s">
         <v>1405</v>
       </c>
-      <c r="D582" s="52" t="s">
+      <c r="D582" s="50" t="s">
         <v>1406</v>
       </c>
       <c r="E582" s="17" t="s">
@@ -22997,8 +23000,8 @@
       <c r="B583" s="16" t="s">
         <v>1407</v>
       </c>
-      <c r="C583" s="52"/>
-      <c r="D583" s="52"/>
+      <c r="C583" s="50"/>
+      <c r="D583" s="50"/>
       <c r="E583" s="17" t="s">
         <v>1323</v>
       </c>
@@ -23019,8 +23022,8 @@
       <c r="B584" s="16" t="s">
         <v>1408</v>
       </c>
-      <c r="C584" s="52"/>
-      <c r="D584" s="52"/>
+      <c r="C584" s="50"/>
+      <c r="D584" s="50"/>
       <c r="E584" s="17" t="s">
         <v>1323</v>
       </c>
@@ -23041,8 +23044,8 @@
       <c r="B585" s="16" t="s">
         <v>1409</v>
       </c>
-      <c r="C585" s="52"/>
-      <c r="D585" s="52"/>
+      <c r="C585" s="50"/>
+      <c r="D585" s="50"/>
       <c r="E585" s="17" t="s">
         <v>1323</v>
       </c>
@@ -23063,8 +23066,8 @@
       <c r="B586" s="16" t="s">
         <v>1410</v>
       </c>
-      <c r="C586" s="52"/>
-      <c r="D586" s="52"/>
+      <c r="C586" s="50"/>
+      <c r="D586" s="50"/>
       <c r="E586" s="17" t="s">
         <v>1323</v>
       </c>
@@ -23111,10 +23114,10 @@
       <c r="B588" s="16" t="s">
         <v>1414</v>
       </c>
-      <c r="C588" s="52" t="s">
+      <c r="C588" s="50" t="s">
         <v>1415</v>
       </c>
-      <c r="D588" s="52" t="s">
+      <c r="D588" s="50" t="s">
         <v>1416</v>
       </c>
       <c r="E588" s="17" t="s">
@@ -23137,8 +23140,8 @@
       <c r="B589" s="16" t="s">
         <v>1417</v>
       </c>
-      <c r="C589" s="52"/>
-      <c r="D589" s="52"/>
+      <c r="C589" s="50"/>
+      <c r="D589" s="50"/>
       <c r="E589" s="17" t="s">
         <v>1323</v>
       </c>
@@ -23211,10 +23214,10 @@
       <c r="B592" s="16" t="s">
         <v>1425</v>
       </c>
-      <c r="C592" s="52" t="s">
+      <c r="C592" s="50" t="s">
         <v>1426</v>
       </c>
-      <c r="D592" s="52" t="s">
+      <c r="D592" s="50" t="s">
         <v>1426</v>
       </c>
       <c r="E592" s="17" t="s">
@@ -23237,8 +23240,8 @@
       <c r="B593" s="16" t="s">
         <v>1427</v>
       </c>
-      <c r="C593" s="52"/>
-      <c r="D593" s="52"/>
+      <c r="C593" s="50"/>
+      <c r="D593" s="50"/>
       <c r="E593" s="17" t="s">
         <v>1323</v>
       </c>
@@ -23259,10 +23262,10 @@
       <c r="B594" s="16" t="s">
         <v>1428</v>
       </c>
-      <c r="C594" s="52" t="s">
+      <c r="C594" s="50" t="s">
         <v>1429</v>
       </c>
-      <c r="D594" s="52" t="s">
+      <c r="D594" s="50" t="s">
         <v>1430</v>
       </c>
       <c r="E594" s="17" t="s">
@@ -23285,8 +23288,8 @@
       <c r="B595" s="16" t="s">
         <v>1431</v>
       </c>
-      <c r="C595" s="52"/>
-      <c r="D595" s="52"/>
+      <c r="C595" s="50"/>
+      <c r="D595" s="50"/>
       <c r="E595" s="17" t="s">
         <v>1323</v>
       </c>
@@ -23307,8 +23310,8 @@
       <c r="B596" s="16" t="s">
         <v>1432</v>
       </c>
-      <c r="C596" s="52"/>
-      <c r="D596" s="52"/>
+      <c r="C596" s="50"/>
+      <c r="D596" s="50"/>
       <c r="E596" s="17" t="s">
         <v>1323</v>
       </c>
@@ -23353,10 +23356,10 @@
       <c r="B598" s="16" t="s">
         <v>1435</v>
       </c>
-      <c r="C598" s="52" t="s">
+      <c r="C598" s="50" t="s">
         <v>1436</v>
       </c>
-      <c r="D598" s="52" t="s">
+      <c r="D598" s="50" t="s">
         <v>1437</v>
       </c>
       <c r="E598" s="17" t="s">
@@ -23379,8 +23382,8 @@
       <c r="B599" s="16" t="s">
         <v>1439</v>
       </c>
-      <c r="C599" s="52"/>
-      <c r="D599" s="52"/>
+      <c r="C599" s="50"/>
+      <c r="D599" s="50"/>
       <c r="E599" s="17" t="s">
         <v>8</v>
       </c>
@@ -23401,8 +23404,8 @@
       <c r="B600" s="16" t="s">
         <v>1440</v>
       </c>
-      <c r="C600" s="52"/>
-      <c r="D600" s="52"/>
+      <c r="C600" s="50"/>
+      <c r="D600" s="50"/>
       <c r="E600" s="17" t="s">
         <v>8</v>
       </c>
@@ -23449,10 +23452,10 @@
       <c r="B602" s="16" t="s">
         <v>1444</v>
       </c>
-      <c r="C602" s="52" t="s">
+      <c r="C602" s="50" t="s">
         <v>1445</v>
       </c>
-      <c r="D602" s="52" t="s">
+      <c r="D602" s="50" t="s">
         <v>1446</v>
       </c>
       <c r="E602" s="17" t="s">
@@ -23475,8 +23478,8 @@
       <c r="B603" s="16" t="s">
         <v>1447</v>
       </c>
-      <c r="C603" s="52"/>
-      <c r="D603" s="52"/>
+      <c r="C603" s="50"/>
+      <c r="D603" s="50"/>
       <c r="E603" s="17" t="s">
         <v>8</v>
       </c>
@@ -23521,10 +23524,10 @@
       <c r="B605" s="16" t="s">
         <v>1450</v>
       </c>
-      <c r="C605" s="52" t="s">
+      <c r="C605" s="50" t="s">
         <v>1451</v>
       </c>
-      <c r="D605" s="52" t="s">
+      <c r="D605" s="50" t="s">
         <v>1452</v>
       </c>
       <c r="E605" s="17" t="s">
@@ -23547,8 +23550,8 @@
       <c r="B606" s="16" t="s">
         <v>1454</v>
       </c>
-      <c r="C606" s="52"/>
-      <c r="D606" s="52"/>
+      <c r="C606" s="50"/>
+      <c r="D606" s="50"/>
       <c r="E606" s="17" t="s">
         <v>8</v>
       </c>
@@ -23569,8 +23572,8 @@
       <c r="B607" s="16" t="s">
         <v>1455</v>
       </c>
-      <c r="C607" s="52"/>
-      <c r="D607" s="52"/>
+      <c r="C607" s="50"/>
+      <c r="D607" s="50"/>
       <c r="E607" s="17" t="s">
         <v>8</v>
       </c>
@@ -23591,8 +23594,8 @@
       <c r="B608" s="16" t="s">
         <v>1456</v>
       </c>
-      <c r="C608" s="52"/>
-      <c r="D608" s="52"/>
+      <c r="C608" s="50"/>
+      <c r="D608" s="50"/>
       <c r="E608" s="17" t="s">
         <v>8</v>
       </c>
@@ -23613,8 +23616,8 @@
       <c r="B609" s="16" t="s">
         <v>1457</v>
       </c>
-      <c r="C609" s="52"/>
-      <c r="D609" s="52"/>
+      <c r="C609" s="50"/>
+      <c r="D609" s="50"/>
       <c r="E609" s="17" t="s">
         <v>8</v>
       </c>
@@ -23635,10 +23638,10 @@
       <c r="B610" s="16" t="s">
         <v>1458</v>
       </c>
-      <c r="C610" s="52" t="s">
+      <c r="C610" s="50" t="s">
         <v>1459</v>
       </c>
-      <c r="D610" s="52" t="s">
+      <c r="D610" s="50" t="s">
         <v>1460</v>
       </c>
       <c r="E610" s="17" t="s">
@@ -23661,8 +23664,8 @@
       <c r="B611" s="16" t="s">
         <v>1462</v>
       </c>
-      <c r="C611" s="52"/>
-      <c r="D611" s="52"/>
+      <c r="C611" s="50"/>
+      <c r="D611" s="50"/>
       <c r="E611" s="17" t="s">
         <v>8</v>
       </c>
@@ -23683,8 +23686,8 @@
       <c r="B612" s="16" t="s">
         <v>1463</v>
       </c>
-      <c r="C612" s="52"/>
-      <c r="D612" s="52"/>
+      <c r="C612" s="50"/>
+      <c r="D612" s="50"/>
       <c r="E612" s="17" t="s">
         <v>8</v>
       </c>
@@ -23705,8 +23708,8 @@
       <c r="B613" s="16" t="s">
         <v>1464</v>
       </c>
-      <c r="C613" s="52"/>
-      <c r="D613" s="52"/>
+      <c r="C613" s="50"/>
+      <c r="D613" s="50"/>
       <c r="E613" s="17" t="s">
         <v>8</v>
       </c>
@@ -23727,8 +23730,8 @@
       <c r="B614" s="16" t="s">
         <v>1465</v>
       </c>
-      <c r="C614" s="52"/>
-      <c r="D614" s="52"/>
+      <c r="C614" s="50"/>
+      <c r="D614" s="50"/>
       <c r="E614" s="17" t="s">
         <v>8</v>
       </c>
@@ -23749,8 +23752,8 @@
       <c r="B615" s="16" t="s">
         <v>1090</v>
       </c>
-      <c r="C615" s="52"/>
-      <c r="D615" s="52"/>
+      <c r="C615" s="50"/>
+      <c r="D615" s="50"/>
       <c r="E615" s="17" t="s">
         <v>8</v>
       </c>
@@ -23948,7 +23951,219 @@
       <c r="F623" s="7"/>
     </row>
   </sheetData>
+  <autoFilter ref="A3:H3" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <mergeCells count="225">
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="D40:D42"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="C13:C21"/>
+    <mergeCell ref="D13:D21"/>
+    <mergeCell ref="C22:C28"/>
+    <mergeCell ref="D22:D28"/>
+    <mergeCell ref="C29:C33"/>
+    <mergeCell ref="D29:D33"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="D67:D68"/>
+    <mergeCell ref="C69:C73"/>
+    <mergeCell ref="D69:D73"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="D51:D52"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="D53:D54"/>
+    <mergeCell ref="C57:C63"/>
+    <mergeCell ref="D57:D63"/>
+    <mergeCell ref="C99:C103"/>
+    <mergeCell ref="D99:D103"/>
+    <mergeCell ref="C104:C106"/>
+    <mergeCell ref="D104:D106"/>
+    <mergeCell ref="C108:C110"/>
+    <mergeCell ref="D108:D110"/>
+    <mergeCell ref="C76:C77"/>
+    <mergeCell ref="D76:D77"/>
+    <mergeCell ref="C88:C89"/>
+    <mergeCell ref="D88:D89"/>
+    <mergeCell ref="C90:C91"/>
+    <mergeCell ref="D90:D91"/>
+    <mergeCell ref="C130:C131"/>
+    <mergeCell ref="D130:D131"/>
+    <mergeCell ref="C144:C145"/>
+    <mergeCell ref="D144:D145"/>
+    <mergeCell ref="C147:C149"/>
+    <mergeCell ref="D147:D149"/>
+    <mergeCell ref="C115:C117"/>
+    <mergeCell ref="D115:D117"/>
+    <mergeCell ref="C118:C119"/>
+    <mergeCell ref="D118:D119"/>
+    <mergeCell ref="C126:C127"/>
+    <mergeCell ref="D126:D127"/>
+    <mergeCell ref="C181:C182"/>
+    <mergeCell ref="D181:D182"/>
+    <mergeCell ref="C183:C185"/>
+    <mergeCell ref="D183:D185"/>
+    <mergeCell ref="C187:C189"/>
+    <mergeCell ref="D187:D189"/>
+    <mergeCell ref="C151:C152"/>
+    <mergeCell ref="D151:D152"/>
+    <mergeCell ref="C163:C164"/>
+    <mergeCell ref="D163:D164"/>
+    <mergeCell ref="C168:C174"/>
+    <mergeCell ref="D168:D174"/>
+    <mergeCell ref="C206:C207"/>
+    <mergeCell ref="D206:D207"/>
+    <mergeCell ref="C209:C210"/>
+    <mergeCell ref="D209:D210"/>
+    <mergeCell ref="C212:C213"/>
+    <mergeCell ref="D212:D213"/>
+    <mergeCell ref="C195:C198"/>
+    <mergeCell ref="D195:D198"/>
+    <mergeCell ref="C200:C201"/>
+    <mergeCell ref="D200:D201"/>
+    <mergeCell ref="C203:C204"/>
+    <mergeCell ref="D203:D204"/>
+    <mergeCell ref="C228:C229"/>
+    <mergeCell ref="D228:D229"/>
+    <mergeCell ref="C232:C234"/>
+    <mergeCell ref="D232:D234"/>
+    <mergeCell ref="C240:C247"/>
+    <mergeCell ref="D240:D247"/>
+    <mergeCell ref="C214:C216"/>
+    <mergeCell ref="D214:D216"/>
+    <mergeCell ref="C217:C218"/>
+    <mergeCell ref="D217:D218"/>
+    <mergeCell ref="C223:C224"/>
+    <mergeCell ref="D223:D224"/>
+    <mergeCell ref="C266:C271"/>
+    <mergeCell ref="D266:D271"/>
+    <mergeCell ref="C273:C274"/>
+    <mergeCell ref="D273:D274"/>
+    <mergeCell ref="C277:C278"/>
+    <mergeCell ref="D277:D278"/>
+    <mergeCell ref="C250:C252"/>
+    <mergeCell ref="D250:D252"/>
+    <mergeCell ref="C258:C259"/>
+    <mergeCell ref="D258:D259"/>
+    <mergeCell ref="C260:C261"/>
+    <mergeCell ref="D260:D261"/>
+    <mergeCell ref="C289:C291"/>
+    <mergeCell ref="D289:D292"/>
+    <mergeCell ref="C293:C296"/>
+    <mergeCell ref="D293:D296"/>
+    <mergeCell ref="C297:C304"/>
+    <mergeCell ref="D297:D304"/>
+    <mergeCell ref="C279:C280"/>
+    <mergeCell ref="D279:D280"/>
+    <mergeCell ref="C281:C282"/>
+    <mergeCell ref="D281:D282"/>
+    <mergeCell ref="C286:C288"/>
+    <mergeCell ref="D286:D288"/>
+    <mergeCell ref="C320:C321"/>
+    <mergeCell ref="D320:D321"/>
+    <mergeCell ref="C324:C325"/>
+    <mergeCell ref="D324:D325"/>
+    <mergeCell ref="C331:C332"/>
+    <mergeCell ref="D331:D332"/>
+    <mergeCell ref="C306:C307"/>
+    <mergeCell ref="D306:D307"/>
+    <mergeCell ref="C308:C309"/>
+    <mergeCell ref="D308:D309"/>
+    <mergeCell ref="C315:C316"/>
+    <mergeCell ref="D315:D316"/>
+    <mergeCell ref="C357:C358"/>
+    <mergeCell ref="D357:D358"/>
+    <mergeCell ref="C359:C360"/>
+    <mergeCell ref="D359:D360"/>
+    <mergeCell ref="C361:C362"/>
+    <mergeCell ref="D361:D362"/>
+    <mergeCell ref="C333:C339"/>
+    <mergeCell ref="D333:D339"/>
+    <mergeCell ref="C343:C344"/>
+    <mergeCell ref="D343:D344"/>
+    <mergeCell ref="C346:C347"/>
+    <mergeCell ref="D346:D347"/>
+    <mergeCell ref="C391:C392"/>
+    <mergeCell ref="D391:D392"/>
+    <mergeCell ref="C393:C394"/>
+    <mergeCell ref="D393:D394"/>
+    <mergeCell ref="C396:C397"/>
+    <mergeCell ref="D396:D397"/>
+    <mergeCell ref="C363:C364"/>
+    <mergeCell ref="D363:D364"/>
+    <mergeCell ref="C370:C372"/>
+    <mergeCell ref="D370:D372"/>
+    <mergeCell ref="C381:C382"/>
+    <mergeCell ref="D381:D382"/>
+    <mergeCell ref="C416:C424"/>
+    <mergeCell ref="D416:D424"/>
+    <mergeCell ref="C429:C430"/>
+    <mergeCell ref="D429:D430"/>
+    <mergeCell ref="C433:C436"/>
+    <mergeCell ref="D433:D436"/>
+    <mergeCell ref="C398:C400"/>
+    <mergeCell ref="D398:D400"/>
+    <mergeCell ref="C401:C405"/>
+    <mergeCell ref="D401:D405"/>
+    <mergeCell ref="C411:C412"/>
+    <mergeCell ref="D411:D412"/>
+    <mergeCell ref="C453:C463"/>
+    <mergeCell ref="D453:D463"/>
+    <mergeCell ref="C469:C470"/>
+    <mergeCell ref="D469:D470"/>
+    <mergeCell ref="C478:C480"/>
+    <mergeCell ref="D478:D480"/>
+    <mergeCell ref="C438:C442"/>
+    <mergeCell ref="D438:D442"/>
+    <mergeCell ref="C444:C445"/>
+    <mergeCell ref="D444:D445"/>
+    <mergeCell ref="C448:C452"/>
+    <mergeCell ref="D448:D452"/>
+    <mergeCell ref="C511:C512"/>
+    <mergeCell ref="D511:D512"/>
+    <mergeCell ref="C514:C515"/>
+    <mergeCell ref="D514:D515"/>
+    <mergeCell ref="C518:C520"/>
+    <mergeCell ref="D518:D520"/>
+    <mergeCell ref="C485:C486"/>
+    <mergeCell ref="D485:D486"/>
+    <mergeCell ref="C497:C498"/>
+    <mergeCell ref="D497:D498"/>
+    <mergeCell ref="C504:C509"/>
+    <mergeCell ref="D504:D509"/>
+    <mergeCell ref="C536:C537"/>
+    <mergeCell ref="D536:D537"/>
+    <mergeCell ref="C541:C542"/>
+    <mergeCell ref="D541:D542"/>
+    <mergeCell ref="C548:C550"/>
+    <mergeCell ref="D548:D550"/>
+    <mergeCell ref="C522:C523"/>
+    <mergeCell ref="D522:D523"/>
+    <mergeCell ref="C526:C529"/>
+    <mergeCell ref="D526:D529"/>
+    <mergeCell ref="C530:C535"/>
+    <mergeCell ref="D530:D535"/>
+    <mergeCell ref="C575:C576"/>
+    <mergeCell ref="D575:D576"/>
+    <mergeCell ref="C577:C578"/>
+    <mergeCell ref="D577:D578"/>
+    <mergeCell ref="C582:C586"/>
+    <mergeCell ref="D582:D586"/>
+    <mergeCell ref="C554:C555"/>
+    <mergeCell ref="D554:D555"/>
+    <mergeCell ref="C557:C569"/>
+    <mergeCell ref="D557:D569"/>
+    <mergeCell ref="C570:C574"/>
+    <mergeCell ref="D570:D574"/>
     <mergeCell ref="C610:C615"/>
     <mergeCell ref="D610:D615"/>
     <mergeCell ref="C598:C600"/>
@@ -23963,217 +24178,6 @@
     <mergeCell ref="D592:D593"/>
     <mergeCell ref="C594:C596"/>
     <mergeCell ref="D594:D596"/>
-    <mergeCell ref="C575:C576"/>
-    <mergeCell ref="D575:D576"/>
-    <mergeCell ref="C577:C578"/>
-    <mergeCell ref="D577:D578"/>
-    <mergeCell ref="C582:C586"/>
-    <mergeCell ref="D582:D586"/>
-    <mergeCell ref="C554:C555"/>
-    <mergeCell ref="D554:D555"/>
-    <mergeCell ref="C557:C569"/>
-    <mergeCell ref="D557:D569"/>
-    <mergeCell ref="C570:C574"/>
-    <mergeCell ref="D570:D574"/>
-    <mergeCell ref="C536:C537"/>
-    <mergeCell ref="D536:D537"/>
-    <mergeCell ref="C541:C542"/>
-    <mergeCell ref="D541:D542"/>
-    <mergeCell ref="C548:C550"/>
-    <mergeCell ref="D548:D550"/>
-    <mergeCell ref="C522:C523"/>
-    <mergeCell ref="D522:D523"/>
-    <mergeCell ref="C526:C529"/>
-    <mergeCell ref="D526:D529"/>
-    <mergeCell ref="C530:C535"/>
-    <mergeCell ref="D530:D535"/>
-    <mergeCell ref="C511:C512"/>
-    <mergeCell ref="D511:D512"/>
-    <mergeCell ref="C514:C515"/>
-    <mergeCell ref="D514:D515"/>
-    <mergeCell ref="C518:C520"/>
-    <mergeCell ref="D518:D520"/>
-    <mergeCell ref="C485:C486"/>
-    <mergeCell ref="D485:D486"/>
-    <mergeCell ref="C497:C498"/>
-    <mergeCell ref="D497:D498"/>
-    <mergeCell ref="C504:C509"/>
-    <mergeCell ref="D504:D509"/>
-    <mergeCell ref="C453:C463"/>
-    <mergeCell ref="D453:D463"/>
-    <mergeCell ref="C469:C470"/>
-    <mergeCell ref="D469:D470"/>
-    <mergeCell ref="C478:C480"/>
-    <mergeCell ref="D478:D480"/>
-    <mergeCell ref="C438:C442"/>
-    <mergeCell ref="D438:D442"/>
-    <mergeCell ref="C444:C445"/>
-    <mergeCell ref="D444:D445"/>
-    <mergeCell ref="C448:C452"/>
-    <mergeCell ref="D448:D452"/>
-    <mergeCell ref="C416:C424"/>
-    <mergeCell ref="D416:D424"/>
-    <mergeCell ref="C429:C430"/>
-    <mergeCell ref="D429:D430"/>
-    <mergeCell ref="C433:C436"/>
-    <mergeCell ref="D433:D436"/>
-    <mergeCell ref="C398:C400"/>
-    <mergeCell ref="D398:D400"/>
-    <mergeCell ref="C401:C405"/>
-    <mergeCell ref="D401:D405"/>
-    <mergeCell ref="C411:C412"/>
-    <mergeCell ref="D411:D412"/>
-    <mergeCell ref="C391:C392"/>
-    <mergeCell ref="D391:D392"/>
-    <mergeCell ref="C393:C394"/>
-    <mergeCell ref="D393:D394"/>
-    <mergeCell ref="C396:C397"/>
-    <mergeCell ref="D396:D397"/>
-    <mergeCell ref="C363:C364"/>
-    <mergeCell ref="D363:D364"/>
-    <mergeCell ref="C370:C372"/>
-    <mergeCell ref="D370:D372"/>
-    <mergeCell ref="C381:C382"/>
-    <mergeCell ref="D381:D382"/>
-    <mergeCell ref="C357:C358"/>
-    <mergeCell ref="D357:D358"/>
-    <mergeCell ref="C359:C360"/>
-    <mergeCell ref="D359:D360"/>
-    <mergeCell ref="C361:C362"/>
-    <mergeCell ref="D361:D362"/>
-    <mergeCell ref="C333:C339"/>
-    <mergeCell ref="D333:D339"/>
-    <mergeCell ref="C343:C344"/>
-    <mergeCell ref="D343:D344"/>
-    <mergeCell ref="C346:C347"/>
-    <mergeCell ref="D346:D347"/>
-    <mergeCell ref="C320:C321"/>
-    <mergeCell ref="D320:D321"/>
-    <mergeCell ref="C324:C325"/>
-    <mergeCell ref="D324:D325"/>
-    <mergeCell ref="C331:C332"/>
-    <mergeCell ref="D331:D332"/>
-    <mergeCell ref="C306:C307"/>
-    <mergeCell ref="D306:D307"/>
-    <mergeCell ref="C308:C309"/>
-    <mergeCell ref="D308:D309"/>
-    <mergeCell ref="C315:C316"/>
-    <mergeCell ref="D315:D316"/>
-    <mergeCell ref="C289:C291"/>
-    <mergeCell ref="D289:D292"/>
-    <mergeCell ref="C293:C296"/>
-    <mergeCell ref="D293:D296"/>
-    <mergeCell ref="C297:C304"/>
-    <mergeCell ref="D297:D304"/>
-    <mergeCell ref="C279:C280"/>
-    <mergeCell ref="D279:D280"/>
-    <mergeCell ref="C281:C282"/>
-    <mergeCell ref="D281:D282"/>
-    <mergeCell ref="C286:C288"/>
-    <mergeCell ref="D286:D288"/>
-    <mergeCell ref="C266:C271"/>
-    <mergeCell ref="D266:D271"/>
-    <mergeCell ref="C273:C274"/>
-    <mergeCell ref="D273:D274"/>
-    <mergeCell ref="C277:C278"/>
-    <mergeCell ref="D277:D278"/>
-    <mergeCell ref="C250:C252"/>
-    <mergeCell ref="D250:D252"/>
-    <mergeCell ref="C258:C259"/>
-    <mergeCell ref="D258:D259"/>
-    <mergeCell ref="C260:C261"/>
-    <mergeCell ref="D260:D261"/>
-    <mergeCell ref="C228:C229"/>
-    <mergeCell ref="D228:D229"/>
-    <mergeCell ref="C232:C234"/>
-    <mergeCell ref="D232:D234"/>
-    <mergeCell ref="C240:C247"/>
-    <mergeCell ref="D240:D247"/>
-    <mergeCell ref="C214:C216"/>
-    <mergeCell ref="D214:D216"/>
-    <mergeCell ref="C217:C218"/>
-    <mergeCell ref="D217:D218"/>
-    <mergeCell ref="C223:C224"/>
-    <mergeCell ref="D223:D224"/>
-    <mergeCell ref="C206:C207"/>
-    <mergeCell ref="D206:D207"/>
-    <mergeCell ref="C209:C210"/>
-    <mergeCell ref="D209:D210"/>
-    <mergeCell ref="C212:C213"/>
-    <mergeCell ref="D212:D213"/>
-    <mergeCell ref="C195:C198"/>
-    <mergeCell ref="D195:D198"/>
-    <mergeCell ref="C200:C201"/>
-    <mergeCell ref="D200:D201"/>
-    <mergeCell ref="C203:C204"/>
-    <mergeCell ref="D203:D204"/>
-    <mergeCell ref="C181:C182"/>
-    <mergeCell ref="D181:D182"/>
-    <mergeCell ref="C183:C185"/>
-    <mergeCell ref="D183:D185"/>
-    <mergeCell ref="C187:C189"/>
-    <mergeCell ref="D187:D189"/>
-    <mergeCell ref="C151:C152"/>
-    <mergeCell ref="D151:D152"/>
-    <mergeCell ref="C163:C164"/>
-    <mergeCell ref="D163:D164"/>
-    <mergeCell ref="C168:C174"/>
-    <mergeCell ref="D168:D174"/>
-    <mergeCell ref="C130:C131"/>
-    <mergeCell ref="D130:D131"/>
-    <mergeCell ref="C144:C145"/>
-    <mergeCell ref="D144:D145"/>
-    <mergeCell ref="C147:C149"/>
-    <mergeCell ref="D147:D149"/>
-    <mergeCell ref="C115:C117"/>
-    <mergeCell ref="D115:D117"/>
-    <mergeCell ref="C118:C119"/>
-    <mergeCell ref="D118:D119"/>
-    <mergeCell ref="C126:C127"/>
-    <mergeCell ref="D126:D127"/>
-    <mergeCell ref="C99:C103"/>
-    <mergeCell ref="D99:D103"/>
-    <mergeCell ref="C104:C106"/>
-    <mergeCell ref="D104:D106"/>
-    <mergeCell ref="C108:C110"/>
-    <mergeCell ref="D108:D110"/>
-    <mergeCell ref="C76:C77"/>
-    <mergeCell ref="D76:D77"/>
-    <mergeCell ref="C88:C89"/>
-    <mergeCell ref="D88:D89"/>
-    <mergeCell ref="C90:C91"/>
-    <mergeCell ref="D90:D91"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="D67:D68"/>
-    <mergeCell ref="C69:C73"/>
-    <mergeCell ref="D69:D73"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="D51:D52"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="D53:D54"/>
-    <mergeCell ref="C57:C63"/>
-    <mergeCell ref="D57:D63"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="D40:D42"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="C13:C21"/>
-    <mergeCell ref="D13:D21"/>
-    <mergeCell ref="C22:C28"/>
-    <mergeCell ref="D22:D28"/>
-    <mergeCell ref="C29:C33"/>
-    <mergeCell ref="D29:D33"/>
-    <mergeCell ref="A1:H2"/>
-    <mergeCell ref="C5:C8"/>
-    <mergeCell ref="D5:D8"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="D37:D38"/>
   </mergeCells>
   <conditionalFormatting sqref="A493:A502">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>